<commit_message>
docs: align Sprint 4 implementation and test ownership
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-4-test-cases.xlsx
+++ b/docs/testing/sprint-4-test-cases.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R30254d41e0544268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R519a2f86dd7c42c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="3" r:id="R72771aa2a7524761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4978b253cba94f93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="Rb01ef5adc3224fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="3" r:id="R3b9b95c28a8b4afd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -138,35 +138,35 @@
   <x:dxfs count="5">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5CD"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDEDED"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -314,7 +314,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9f7ef14a1db14170"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1bd52442eb549fe"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1082,13 +1082,57 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>Test Owner</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Assigned Tests</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="B26" t="n">
+        <x:f>COUNTIF('Test Cases'!$K$6:$K$134,A26)</x:f>
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>MD</x:v>
+      </x:c>
+      <x:c r="B27" t="n">
+        <x:f>COUNTIF('Test Cases'!$K$6:$K$134,A27)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>Joyee</x:v>
+      </x:c>
+      <x:c r="B28" t="n">
+        <x:f>COUNTIF('Test Cases'!$K$6:$K$134,A28)</x:f>
+        <x:v>45</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>Total</x:v>
+      </x:c>
+      <x:c r="B29" t="n">
+        <x:f>SUM(B26:B28)</x:f>
+        <x:v>129</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7215074b45c14153"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb66c4c55c93f489e"/>
 </x:worksheet>
 </file>
 
@@ -1248,7 +1292,7 @@
         <x:v>Backend reaches the configured PostgreSQL database without connection error.</x:v>
       </x:c>
       <x:c r="K6" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L6" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1294,7 +1338,7 @@
         <x:v>Django reports no system-check issues.</x:v>
       </x:c>
       <x:c r="K7" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L7" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1340,7 +1384,7 @@
         <x:v>No uncommitted model changes require a new migration.</x:v>
       </x:c>
       <x:c r="K8" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L8" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1386,7 +1430,7 @@
         <x:v>Full backend suite passes with no failures or errors.</x:v>
       </x:c>
       <x:c r="K9" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L9" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -1434,7 +1478,7 @@
         <x:v>Lint completes with no errors.</x:v>
       </x:c>
       <x:c r="K10" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L10" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1480,7 +1524,7 @@
         <x:v>Production build completes successfully.</x:v>
       </x:c>
       <x:c r="K11" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L11" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1526,7 +1570,7 @@
         <x:v>Local integration baseline matches origin/feature/sprint-4.</x:v>
       </x:c>
       <x:c r="K12" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L12" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -1574,7 +1618,7 @@
         <x:v>Student is authenticated and routed to the protected Student application.</x:v>
       </x:c>
       <x:c r="K13" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L13" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1620,7 +1664,7 @@
         <x:v>Login is rejected with a controlled validation or authentication message.</x:v>
       </x:c>
       <x:c r="K14" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L14" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1666,7 +1710,7 @@
         <x:v>Access is blocked and the user is directed to authentication.</x:v>
       </x:c>
       <x:c r="K15" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L15" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1712,7 +1756,7 @@
         <x:v>API rejects the request with the approved unauthenticated response.</x:v>
       </x:c>
       <x:c r="K16" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L16" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1758,7 +1802,7 @@
         <x:v>Authenticated Student identity is returned without exposing sensitive fields.</x:v>
       </x:c>
       <x:c r="K17" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L17" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1804,7 +1848,7 @@
         <x:v>Only the authenticated Student profile loads.</x:v>
       </x:c>
       <x:c r="K18" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L18" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1850,7 +1894,7 @@
         <x:v>Update persists and reloads correctly.</x:v>
       </x:c>
       <x:c r="K19" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L19" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1896,7 +1940,7 @@
         <x:v>Backend prevents cross-student access.</x:v>
       </x:c>
       <x:c r="K20" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L20" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1942,7 +1986,7 @@
         <x:v>Dependent feature uses the updated authenticated Student context.</x:v>
       </x:c>
       <x:c r="K21" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L21" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -1988,7 +2032,7 @@
         <x:v>Ranked deterministic recommendations are returned.</x:v>
       </x:c>
       <x:c r="K22" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L22" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2034,7 +2078,7 @@
         <x:v>Recommendation score is displayed with the result.</x:v>
       </x:c>
       <x:c r="K23" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L23" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2053,7 +2097,7 @@
         <x:v>S4-REC-03</x:v>
       </x:c>
       <x:c r="B24" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.4,7.9</x:v>
       </x:c>
       <x:c r="C24" s="28" t="str">
         <x:v>Career Recommendations</x:v>
@@ -2080,7 +2124,7 @@
         <x:v>Explanation is returned without changing deterministic score or rank.</x:v>
       </x:c>
       <x:c r="K24" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L24" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -2128,7 +2172,7 @@
         <x:v>Deterministic recommendation order and scores repeat.</x:v>
       </x:c>
       <x:c r="K25" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L25" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2174,7 +2218,7 @@
         <x:v>Each Student receives results from their own profile context.</x:v>
       </x:c>
       <x:c r="K26" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L26" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2193,7 +2237,7 @@
         <x:v>S4-REC-06</x:v>
       </x:c>
       <x:c r="B27" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.4,7.9</x:v>
       </x:c>
       <x:c r="C27" s="28" t="str">
         <x:v>Career Recommendations</x:v>
@@ -2220,7 +2264,7 @@
         <x:v>Deterministic recommendation score and rank remain unchanged.</x:v>
       </x:c>
       <x:c r="K27" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L27" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -2268,7 +2312,7 @@
         <x:v>Matched and missing requirements are shown for the selected Career.</x:v>
       </x:c>
       <x:c r="K28" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L28" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2314,7 +2358,7 @@
         <x:v>Deterministic readiness score and factor details are returned.</x:v>
       </x:c>
       <x:c r="K29" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L29" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2360,7 +2404,7 @@
         <x:v>Deterministic results repeat.</x:v>
       </x:c>
       <x:c r="K30" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L30" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2379,7 +2423,7 @@
         <x:v>S4-GAP-04</x:v>
       </x:c>
       <x:c r="B31" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.4,7.9</x:v>
       </x:c>
       <x:c r="C31" s="28" t="str">
         <x:v>Skill Gap and Readiness</x:v>
@@ -2406,7 +2450,7 @@
         <x:v>Deterministic matched and missing requirements remain unchanged.</x:v>
       </x:c>
       <x:c r="K31" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L31" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -2427,7 +2471,7 @@
         <x:v>S4-GAP-05</x:v>
       </x:c>
       <x:c r="B32" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.4,7.9</x:v>
       </x:c>
       <x:c r="C32" s="28" t="str">
         <x:v>Skill Gap and Readiness</x:v>
@@ -2454,7 +2498,7 @@
         <x:v>Readiness deterministic response remains available.</x:v>
       </x:c>
       <x:c r="K32" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L32" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2500,7 +2544,7 @@
         <x:v>Ranked resources load for unresolved skill gaps.</x:v>
       </x:c>
       <x:c r="K33" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L33" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2546,7 +2590,7 @@
         <x:v>Resources reflect the active selected Career context.</x:v>
       </x:c>
       <x:c r="K34" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L34" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2592,7 +2636,7 @@
         <x:v>Feedback request is handled without breaking the resource list.</x:v>
       </x:c>
       <x:c r="K35" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L35" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2638,7 +2682,7 @@
         <x:v>Report is handled through the approved backend flow.</x:v>
       </x:c>
       <x:c r="K36" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L36" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2684,7 +2728,7 @@
         <x:v>Ordered roadmap steps load for the selected Career.</x:v>
       </x:c>
       <x:c r="K37" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L37" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2730,7 +2774,7 @@
         <x:v>Progress state updates for the authenticated Student.</x:v>
       </x:c>
       <x:c r="K38" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L38" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2776,7 +2820,7 @@
         <x:v>Completion persists and progress updates.</x:v>
       </x:c>
       <x:c r="K39" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L39" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2822,7 +2866,7 @@
         <x:v>Backend prevents cross-student access.</x:v>
       </x:c>
       <x:c r="K40" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L40" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2841,7 +2885,7 @@
         <x:v>S4-JOB-01</x:v>
       </x:c>
       <x:c r="B41" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.5,7.9</x:v>
       </x:c>
       <x:c r="C41" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -2868,7 +2912,7 @@
         <x:v>Job Matching page loads for the authenticated Student.</x:v>
       </x:c>
       <x:c r="K41" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L41" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2887,7 +2931,7 @@
         <x:v>S4-JOB-02</x:v>
       </x:c>
       <x:c r="B42" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.5,7.9</x:v>
       </x:c>
       <x:c r="C42" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -2914,7 +2958,7 @@
         <x:v>Structured matched and missing requirement result is displayed.</x:v>
       </x:c>
       <x:c r="K42" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L42" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2933,7 +2977,7 @@
         <x:v>S4-JOB-03</x:v>
       </x:c>
       <x:c r="B43" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.5,7.9</x:v>
       </x:c>
       <x:c r="C43" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -2960,7 +3004,7 @@
         <x:v>Validation prevents the request or API rejects the blank value.</x:v>
       </x:c>
       <x:c r="K43" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L43" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -2979,7 +3023,7 @@
         <x:v>S4-JOB-04</x:v>
       </x:c>
       <x:c r="B44" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.5,7.9</x:v>
       </x:c>
       <x:c r="C44" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3006,7 +3050,7 @@
         <x:v>Oversized input is rejected with controlled validation.</x:v>
       </x:c>
       <x:c r="K44" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L44" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3025,7 +3069,7 @@
         <x:v>S4-JOB-05</x:v>
       </x:c>
       <x:c r="B45" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.5,7.9</x:v>
       </x:c>
       <x:c r="C45" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3052,7 +3096,7 @@
         <x:v>Known requirements appear in the matched section.</x:v>
       </x:c>
       <x:c r="K45" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L45" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3071,7 +3115,7 @@
         <x:v>S4-JOB-06</x:v>
       </x:c>
       <x:c r="B46" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.5,7.9</x:v>
       </x:c>
       <x:c r="C46" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3098,7 +3142,7 @@
         <x:v>Recognised absent requirements appear in the missing section.</x:v>
       </x:c>
       <x:c r="K46" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L46" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3117,7 +3161,7 @@
         <x:v>S4-JOB-07</x:v>
       </x:c>
       <x:c r="B47" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.9</x:v>
       </x:c>
       <x:c r="C47" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3144,7 +3188,7 @@
         <x:v>Canonical Skill is recognised correctly.</x:v>
       </x:c>
       <x:c r="K47" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L47" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3163,7 +3207,7 @@
         <x:v>S4-JOB-08</x:v>
       </x:c>
       <x:c r="B48" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.9</x:v>
       </x:c>
       <x:c r="C48" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3190,7 +3234,7 @@
         <x:v>Alias resolves to the canonical Skill.</x:v>
       </x:c>
       <x:c r="K48" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L48" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3209,7 +3253,7 @@
         <x:v>S4-JOB-09</x:v>
       </x:c>
       <x:c r="B49" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.9</x:v>
       </x:c>
       <x:c r="C49" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3236,7 +3280,7 @@
         <x:v>Unsupported wording is not silently mapped to a different Skill.</x:v>
       </x:c>
       <x:c r="K49" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L49" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3255,7 +3299,7 @@
         <x:v>S4-JOB-10</x:v>
       </x:c>
       <x:c r="B50" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.9</x:v>
       </x:c>
       <x:c r="C50" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3282,7 +3326,7 @@
         <x:v>Generic wording does not incorrectly map to the canonical Design concept.</x:v>
       </x:c>
       <x:c r="K50" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L50" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3301,7 +3345,7 @@
         <x:v>S4-JOB-11</x:v>
       </x:c>
       <x:c r="B51" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.9</x:v>
       </x:c>
       <x:c r="C51" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3328,7 +3372,7 @@
         <x:v>No hiring probability or employment suitability score is presented.</x:v>
       </x:c>
       <x:c r="K51" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L51" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3347,7 +3391,7 @@
         <x:v>S4-JOB-12</x:v>
       </x:c>
       <x:c r="B52" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.9</x:v>
       </x:c>
       <x:c r="C52" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3374,7 +3418,7 @@
         <x:v>Request is rejected or ownership fields are ignored according to the approved contract.</x:v>
       </x:c>
       <x:c r="K52" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L52" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3393,7 +3437,7 @@
         <x:v>S4-JOB-13</x:v>
       </x:c>
       <x:c r="B53" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.2,7.9</x:v>
       </x:c>
       <x:c r="C53" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3420,7 +3464,7 @@
         <x:v>Student Profile is not mutated by the job-match operation.</x:v>
       </x:c>
       <x:c r="K53" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L53" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3439,7 +3483,7 @@
         <x:v>S4-JOB-14</x:v>
       </x:c>
       <x:c r="B54" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.5,7.9</x:v>
       </x:c>
       <x:c r="C54" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3466,7 +3510,7 @@
         <x:v>Resume Builder receives the current job description context where supported.</x:v>
       </x:c>
       <x:c r="K54" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L54" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3485,7 +3529,7 @@
         <x:v>S4-JOB-15</x:v>
       </x:c>
       <x:c r="B55" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.5,7.9</x:v>
       </x:c>
       <x:c r="C55" s="28" t="str">
         <x:v>Job Matching</x:v>
@@ -3512,7 +3556,7 @@
         <x:v>Cover Letter Builder receives the current job description context.</x:v>
       </x:c>
       <x:c r="K55" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L55" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3558,7 +3602,7 @@
         <x:v>Protected Resume Builder loads.</x:v>
       </x:c>
       <x:c r="K56" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L56" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3577,7 +3621,7 @@
         <x:v>S4-RESUME-02</x:v>
       </x:c>
       <x:c r="B57" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.3,7.9</x:v>
       </x:c>
       <x:c r="C57" s="28" t="str">
         <x:v>Resume Builder</x:v>
@@ -3604,7 +3648,7 @@
         <x:v>Structured Resume draft is returned through the backend provider path.</x:v>
       </x:c>
       <x:c r="K57" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L57" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3650,7 +3694,7 @@
         <x:v>Student edits are accepted in the UI.</x:v>
       </x:c>
       <x:c r="K58" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L58" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3696,7 +3740,7 @@
         <x:v>Draft is presented for user review before use.</x:v>
       </x:c>
       <x:c r="K59" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L59" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3715,7 +3759,7 @@
         <x:v>S4-RESUME-05</x:v>
       </x:c>
       <x:c r="B60" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.4,7.9</x:v>
       </x:c>
       <x:c r="C60" s="28" t="str">
         <x:v>Resume Builder</x:v>
@@ -3742,7 +3786,7 @@
         <x:v>Controlled error is returned without provider internals.</x:v>
       </x:c>
       <x:c r="K60" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L60" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -3763,7 +3807,7 @@
         <x:v>S4-RESUME-06</x:v>
       </x:c>
       <x:c r="B61" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.4,7.9</x:v>
       </x:c>
       <x:c r="C61" s="28" t="str">
         <x:v>Resume Builder</x:v>
@@ -3790,7 +3834,7 @@
         <x:v>Invalid response is rejected and no invalid draft is accepted.</x:v>
       </x:c>
       <x:c r="K61" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L61" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -3811,7 +3855,7 @@
         <x:v>S4-RESUME-07</x:v>
       </x:c>
       <x:c r="B62" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.5,7.9</x:v>
       </x:c>
       <x:c r="C62" s="28" t="str">
         <x:v>Resume Builder</x:v>
@@ -3838,7 +3882,7 @@
         <x:v>Expected job-description context is retained where supported.</x:v>
       </x:c>
       <x:c r="K62" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L62" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3884,7 +3928,7 @@
         <x:v>Protected Cover Letter Builder loads.</x:v>
       </x:c>
       <x:c r="K63" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L63" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3930,7 +3974,7 @@
         <x:v>Generation is prevented with controlled validation.</x:v>
       </x:c>
       <x:c r="K64" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L64" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -3949,7 +3993,7 @@
         <x:v>S4-COVER-03</x:v>
       </x:c>
       <x:c r="B65" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.3,7.9</x:v>
       </x:c>
       <x:c r="C65" s="28" t="str">
         <x:v>Cover Letter Builder</x:v>
@@ -3976,7 +4020,7 @@
         <x:v>Structured Cover Letter draft is returned.</x:v>
       </x:c>
       <x:c r="K65" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L65" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4022,7 +4066,7 @@
         <x:v>Student edits are accepted in the UI.</x:v>
       </x:c>
       <x:c r="K66" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L66" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4068,7 +4112,7 @@
         <x:v>Draft is presented for user review before use.</x:v>
       </x:c>
       <x:c r="K67" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L67" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4087,7 +4131,7 @@
         <x:v>S4-COVER-06</x:v>
       </x:c>
       <x:c r="B68" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.4,7.9</x:v>
       </x:c>
       <x:c r="C68" s="28" t="str">
         <x:v>Cover Letter Builder</x:v>
@@ -4114,7 +4158,7 @@
         <x:v>Controlled error is returned without provider internals.</x:v>
       </x:c>
       <x:c r="K68" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L68" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4135,7 +4179,7 @@
         <x:v>S4-COVER-07</x:v>
       </x:c>
       <x:c r="B69" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.5,7.9</x:v>
       </x:c>
       <x:c r="C69" s="28" t="str">
         <x:v>Cover Letter Builder</x:v>
@@ -4162,7 +4206,7 @@
         <x:v>Current job-description context is carried into the builder.</x:v>
       </x:c>
       <x:c r="K69" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L69" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4208,7 +4252,7 @@
         <x:v>Protected Interview page loads.</x:v>
       </x:c>
       <x:c r="K70" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L70" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4227,7 +4271,7 @@
         <x:v>S4-INT-02</x:v>
       </x:c>
       <x:c r="B71" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.3,7.9</x:v>
       </x:c>
       <x:c r="C71" s="28" t="str">
         <x:v>Interview Preparation</x:v>
@@ -4254,7 +4298,7 @@
         <x:v>Structured Interview Questions are returned.</x:v>
       </x:c>
       <x:c r="K71" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L71" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4300,7 +4344,7 @@
         <x:v>Validation rejects the request.</x:v>
       </x:c>
       <x:c r="K72" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L72" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4346,7 +4390,7 @@
         <x:v>Validation rejects the request.</x:v>
       </x:c>
       <x:c r="K73" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L73" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4392,7 +4436,7 @@
         <x:v>Returned questions render correctly.</x:v>
       </x:c>
       <x:c r="K74" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L74" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4438,7 +4482,7 @@
         <x:v>Answer is accepted as untrusted user input.</x:v>
       </x:c>
       <x:c r="K75" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L75" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4457,7 +4501,7 @@
         <x:v>S4-INT-07</x:v>
       </x:c>
       <x:c r="B76" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.3,7.9</x:v>
       </x:c>
       <x:c r="C76" s="28" t="str">
         <x:v>Interview Preparation</x:v>
@@ -4484,7 +4528,7 @@
         <x:v>Structured strengths and improvement feedback is returned.</x:v>
       </x:c>
       <x:c r="K76" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L76" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4503,7 +4547,7 @@
         <x:v>S4-INT-08</x:v>
       </x:c>
       <x:c r="B77" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.4,7.9</x:v>
       </x:c>
       <x:c r="C77" s="28" t="str">
         <x:v>Interview Preparation</x:v>
@@ -4530,7 +4574,7 @@
         <x:v>Semantic validator rejects invalid question set.</x:v>
       </x:c>
       <x:c r="K77" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L77" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4578,7 +4622,7 @@
         <x:v>No hiring probability or pass-fail hiring classification appears.</x:v>
       </x:c>
       <x:c r="K78" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L78" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -4624,7 +4668,7 @@
         <x:v>Completed response proceeds to structured validation.</x:v>
       </x:c>
       <x:c r="K79" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L79" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4672,7 +4716,7 @@
         <x:v>Incomplete response is rejected.</x:v>
       </x:c>
       <x:c r="K80" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L80" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4720,7 +4764,7 @@
         <x:v>Failed response is rejected.</x:v>
       </x:c>
       <x:c r="K81" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L81" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4768,7 +4812,7 @@
         <x:v>Cancelled response is rejected.</x:v>
       </x:c>
       <x:c r="K82" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L82" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4816,7 +4860,7 @@
         <x:v>Non-completed response is rejected.</x:v>
       </x:c>
       <x:c r="K83" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L83" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4864,7 +4908,7 @@
         <x:v>Missing response status is rejected.</x:v>
       </x:c>
       <x:c r="K84" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L84" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4912,7 +4956,7 @@
         <x:v>Empty output is rejected.</x:v>
       </x:c>
       <x:c r="K85" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L85" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -4960,7 +5004,7 @@
         <x:v>Malformed JSON is rejected.</x:v>
       </x:c>
       <x:c r="K86" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L86" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5008,7 +5052,7 @@
         <x:v>Controlled application error is returned without internal detail.</x:v>
       </x:c>
       <x:c r="K87" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L87" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5056,7 +5100,7 @@
         <x:v>Controlled application error is returned without provider internals.</x:v>
       </x:c>
       <x:c r="K88" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L88" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5104,7 +5148,7 @@
         <x:v>Controlled application error is returned without provider internals.</x:v>
       </x:c>
       <x:c r="K89" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L89" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5152,7 +5196,7 @@
         <x:v>Deterministic values remain unchanged.</x:v>
       </x:c>
       <x:c r="K90" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L90" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5200,7 +5244,7 @@
         <x:v>Request is rejected.</x:v>
       </x:c>
       <x:c r="K91" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L91" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5248,7 +5292,7 @@
         <x:v>Backend returns permission denial.</x:v>
       </x:c>
       <x:c r="K92" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L92" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5296,7 +5340,7 @@
         <x:v>Approved administration data is returned.</x:v>
       </x:c>
       <x:c r="K93" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L93" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5344,7 +5388,7 @@
         <x:v>User list excludes password values and unnecessary private profile data.</x:v>
       </x:c>
       <x:c r="K94" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L94" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5392,7 +5436,7 @@
         <x:v>Approved user administration fields are returned.</x:v>
       </x:c>
       <x:c r="K95" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L95" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5440,7 +5484,7 @@
         <x:v>Update succeeds and persists.</x:v>
       </x:c>
       <x:c r="K96" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L96" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5488,7 +5532,7 @@
         <x:v>Career administration follows the approved API contract.</x:v>
       </x:c>
       <x:c r="K97" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L97" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5536,7 +5580,7 @@
         <x:v>Skill administration follows the approved API contract.</x:v>
       </x:c>
       <x:c r="K98" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L98" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5584,7 +5628,7 @@
         <x:v>Learning Resource administration follows the approved API contract.</x:v>
       </x:c>
       <x:c r="K99" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L99" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5632,7 +5676,7 @@
         <x:v>Assignment persists and is returned correctly.</x:v>
       </x:c>
       <x:c r="K100" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L100" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5680,7 +5724,7 @@
         <x:v>Unauthenticated access is blocked.</x:v>
       </x:c>
       <x:c r="K101" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L101" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5728,7 +5772,7 @@
         <x:v>Student cannot use the admin dashboard.</x:v>
       </x:c>
       <x:c r="K102" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L102" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5776,7 +5820,7 @@
         <x:v>Admin Dashboard loads.</x:v>
       </x:c>
       <x:c r="K103" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L103" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5824,7 +5868,7 @@
         <x:v>Loading state is visible while data is pending.</x:v>
       </x:c>
       <x:c r="K104" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L104" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5872,7 +5916,7 @@
         <x:v>Controlled error state is shown.</x:v>
       </x:c>
       <x:c r="K105" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L105" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5920,7 +5964,7 @@
         <x:v>Approved summary information is rendered.</x:v>
       </x:c>
       <x:c r="K106" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L106" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -5968,7 +6012,7 @@
         <x:v>Screen loads and connects to the approved admin API.</x:v>
       </x:c>
       <x:c r="K107" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L107" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6016,7 +6060,7 @@
         <x:v>Backend still rejects the operation.</x:v>
       </x:c>
       <x:c r="K108" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L108" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6064,7 +6108,7 @@
         <x:v>Backend permits the approved role operation.</x:v>
       </x:c>
       <x:c r="K109" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L109" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6112,7 +6156,7 @@
         <x:v>Backend denies access.</x:v>
       </x:c>
       <x:c r="K110" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L110" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6160,7 +6204,7 @@
         <x:v>Backend denies access and no mutation occurs.</x:v>
       </x:c>
       <x:c r="K111" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L111" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6208,7 +6252,7 @@
         <x:v>Request is rejected as unauthenticated.</x:v>
       </x:c>
       <x:c r="K112" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L112" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6256,7 +6300,7 @@
         <x:v>Backend permission enforcement prevents access.</x:v>
       </x:c>
       <x:c r="K113" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L113" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6304,7 +6348,7 @@
         <x:v>Cross-student access remains denied.</x:v>
       </x:c>
       <x:c r="K114" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L114" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6352,7 +6396,7 @@
         <x:v>Required audit record is created.</x:v>
       </x:c>
       <x:c r="K115" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L115" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6400,7 +6444,7 @@
         <x:v>Record identifies the approved action using the required fields.</x:v>
       </x:c>
       <x:c r="K116" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L116" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6448,7 +6492,7 @@
         <x:v>No password or password hash is stored in audit details.</x:v>
       </x:c>
       <x:c r="K117" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L117" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6496,7 +6540,7 @@
         <x:v>No JWT, API key, or secret value is stored.</x:v>
       </x:c>
       <x:c r="K118" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L118" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6544,7 +6588,7 @@
         <x:v>Only approved audit data is retained.</x:v>
       </x:c>
       <x:c r="K119" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L119" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6592,7 +6636,7 @@
         <x:v>Only the approved role has audit access.</x:v>
       </x:c>
       <x:c r="K120" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L120" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6613,7 +6657,7 @@
         <x:v>S4-FE-01</x:v>
       </x:c>
       <x:c r="B121" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.5,7.9</x:v>
       </x:c>
       <x:c r="C121" s="28" t="str">
         <x:v>Frontend Quality</x:v>
@@ -6640,7 +6684,7 @@
         <x:v>Content and actions remain readable and usable.</x:v>
       </x:c>
       <x:c r="K121" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L121" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -6659,7 +6703,7 @@
         <x:v>S4-FE-02</x:v>
       </x:c>
       <x:c r="B122" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.5,7.9</x:v>
       </x:c>
       <x:c r="C122" s="28" t="str">
         <x:v>Frontend Quality</x:v>
@@ -6686,7 +6730,7 @@
         <x:v>Core controls and results remain usable without unintended overflow.</x:v>
       </x:c>
       <x:c r="K122" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L122" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -6705,7 +6749,7 @@
         <x:v>S4-FE-03</x:v>
       </x:c>
       <x:c r="B123" s="28" t="str">
-        <x:v>7.9</x:v>
+        <x:v>7.7,7.9</x:v>
       </x:c>
       <x:c r="C123" s="28" t="str">
         <x:v>Frontend Quality</x:v>
@@ -6732,7 +6776,7 @@
         <x:v>Approved admin dashboard remains usable across planned widths.</x:v>
       </x:c>
       <x:c r="K123" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L123" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6780,7 +6824,7 @@
         <x:v>Interactive controls are reachable in a logical order.</x:v>
       </x:c>
       <x:c r="K124" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L124" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -6826,7 +6870,7 @@
         <x:v>Inputs have meaningful labels and useful validation feedback.</x:v>
       </x:c>
       <x:c r="K125" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L125" s="28" t="str">
         <x:v>Not Run</x:v>
@@ -6872,7 +6916,7 @@
         <x:v>Core flow works in current Chrome.</x:v>
       </x:c>
       <x:c r="K126" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L126" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6920,7 +6964,7 @@
         <x:v>Core flow works in current Edge.</x:v>
       </x:c>
       <x:c r="K127" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L127" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -6968,7 +7012,7 @@
         <x:v>Core flow works in current Firefox.</x:v>
       </x:c>
       <x:c r="K128" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Joyee</x:v>
       </x:c>
       <x:c r="L128" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -7016,7 +7060,7 @@
         <x:v>Core authentication remains working.</x:v>
       </x:c>
       <x:c r="K129" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L129" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -7064,7 +7108,7 @@
         <x:v>Core Student Profile remains working.</x:v>
       </x:c>
       <x:c r="K130" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L130" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -7112,7 +7156,7 @@
         <x:v>Core Sprint 2 career-analysis functions remain working.</x:v>
       </x:c>
       <x:c r="K131" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L131" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -7160,7 +7204,7 @@
         <x:v>Core document flows remain working.</x:v>
       </x:c>
       <x:c r="K132" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>MD</x:v>
       </x:c>
       <x:c r="L132" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -7208,7 +7252,7 @@
         <x:v>Core Interview flow remains working.</x:v>
       </x:c>
       <x:c r="K133" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L133" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -7256,7 +7300,7 @@
         <x:v>Core Sprint 4 integrated increment works without unresolved Critical or High blocking defect.</x:v>
       </x:c>
       <x:c r="K134" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L134" s="28" t="str">
         <x:v>Blocked</x:v>
@@ -7302,7 +7346,7 @@
       <x:formula1>"Unit,Schema,API,Integration,Permission,Security,Frontend,Regression"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K6:K134">
-      <x:formula1>"All Members,Jerald,MD,Joyee"</x:formula1>
+      <x:formula1>"Jerald,MD,Joyee"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L6:L134">
       <x:formula1>"Pass,Fail,Blocked,Not Run,Retest"</x:formula1>
@@ -7313,7 +7357,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb92f86a170fa4412"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196476165ba04ed0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7726,7 +7770,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3de33b97812b41b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b8b3ea5bf074d0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
test: add Sprint 4 WIP execution evidence
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-4-test-cases.xlsx
+++ b/docs/testing/sprint-4-test-cases.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4978b253cba94f93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="Rb01ef5adc3224fcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="3" r:id="R3b9b95c28a8b4afd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc84b0008d5234542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R3029775b09ca4b2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="3" r:id="Rdfbdfce8f3d44a3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,7 +68,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -131,6 +131,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -314,7 +315,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1bd52442eb549fe"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R93e99f05a9df4634"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -586,7 +587,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="13" t="str">
-        <x:v>WBS 7.9 Sprint 4 Integration and Testing. Planning tracker only. Pass and Fail stay at zero until execution.</x:v>
+        <x:v>WBS 7.9 Sprint 4 Integration and Testing. Active execution dashboard. WBS 7.4, 7.5, 7.6, and 7.8 are integrated. Only WBS 7.7-dependent cases remain blocked.</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -633,15 +634,15 @@
         <x:v>Environment</x:v>
       </x:c>
       <x:c r="E5" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D5)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D5)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="F5" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D5,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D5,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G5" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D5,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D5,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="H5" s="28" t="n">
@@ -655,27 +656,27 @@
       </x:c>
       <x:c r="B6" s="28" t="n">
         <x:f>COUNTIF('Test Cases'!L6:L134,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C6" s="28"/>
       <x:c r="D6" s="28" t="str">
         <x:v>Authentication</x:v>
       </x:c>
       <x:c r="E6" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D6)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D6)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F6" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D6,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D6,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D6,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>5</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D6,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H6" s="28" t="n">
         <x:f>E6-F6-G6</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -691,20 +692,20 @@
         <x:v>Student Profile</x:v>
       </x:c>
       <x:c r="E7" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D7)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D7)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F7" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D7,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D7,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D7,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>4</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D7,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H7" s="28" t="n">
         <x:f>E7-F7-G7</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -713,27 +714,27 @@
       </x:c>
       <x:c r="B8" s="28" t="n">
         <x:f>COUNTIF('Test Cases'!L6:L134,"Blocked")</x:f>
-        <x:v>61</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C8" s="28"/>
       <x:c r="D8" s="28" t="str">
         <x:v>Career Recommendations</x:v>
       </x:c>
       <x:c r="E8" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D8)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D8)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F8" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D8,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D8,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="28" t="n">
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D8,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>2</x:v>
-      </x:c>
-      <x:c r="G8" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D8,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>4</x:v>
       </x:c>
       <x:c r="H8" s="28" t="n">
         <x:f>E8-F8-G8</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -749,20 +750,20 @@
         <x:v>Skill Gap and Readiness</x:v>
       </x:c>
       <x:c r="E9" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D9)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D9)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F9" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D9,'Test Cases'!L6:L134,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D9,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D9,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>4</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D9,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H9" s="28" t="n">
         <x:f>E9-F9-G9</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -778,15 +779,15 @@
         <x:v>Learning Suggestions</x:v>
       </x:c>
       <x:c r="E10" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D10)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D10)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F10" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D10,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D10,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D10,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D10,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="H10" s="28" t="n">
@@ -802,15 +803,15 @@
         <x:v>Career Roadmap</x:v>
       </x:c>
       <x:c r="E11" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D11)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D11)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F11" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D11,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D11,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D11,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D11,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="H11" s="28" t="n">
@@ -826,20 +827,20 @@
         <x:v>Job Matching</x:v>
       </x:c>
       <x:c r="E12" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D12)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D12)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="F12" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D12,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D12,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D12,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D12,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H12" s="28" t="n">
         <x:f>E12-F12-G12</x:f>
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -850,20 +851,20 @@
         <x:v>Resume Builder</x:v>
       </x:c>
       <x:c r="E13" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D13)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D13)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="F13" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D13,'Test Cases'!L6:L134,"Blocked")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D13,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D13,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D13,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="H13" s="28" t="n">
         <x:f>E13-F13-G13</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -874,20 +875,20 @@
         <x:v>Cover Letter Builder</x:v>
       </x:c>
       <x:c r="E14" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D14)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D14)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="F14" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D14,'Test Cases'!L6:L134,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D14,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D14,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D14,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="H14" s="28" t="n">
         <x:f>E14-F14-G14</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -898,20 +899,20 @@
         <x:v>Interview Preparation</x:v>
       </x:c>
       <x:c r="E15" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D15)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D15)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="F15" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D15,'Test Cases'!L6:L134,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D15,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D15,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D15,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H15" s="28" t="n">
         <x:f>E15-F15-G15</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -922,20 +923,20 @@
         <x:v>AI Response Validation</x:v>
       </x:c>
       <x:c r="E16" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D16)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D16)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="F16" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D16,'Test Cases'!L6:L134,"Blocked")</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D16,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D16,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D16,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H16" s="28" t="n">
         <x:f>E16-F16-G16</x:f>
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -946,16 +947,16 @@
         <x:v>Admin API</x:v>
       </x:c>
       <x:c r="E17" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D17)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D17)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="F17" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D17,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D17,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" s="28" t="n">
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D17,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>10</x:v>
-      </x:c>
-      <x:c r="G17" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D17,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="H17" s="28" t="n">
         <x:f>E17-F17-G17</x:f>
@@ -970,15 +971,15 @@
         <x:v>Admin Dashboard</x:v>
       </x:c>
       <x:c r="E18" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D18)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D18)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F18" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D18,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D18,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="G18" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D18,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D18,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H18" s="28" t="n">
@@ -994,16 +995,16 @@
         <x:v>Role Permissions</x:v>
       </x:c>
       <x:c r="E19" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D19)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D19)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F19" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D19,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D19,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="28" t="n">
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D19,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>6</x:v>
-      </x:c>
-      <x:c r="G19" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D19,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="H19" s="28" t="n">
         <x:f>E19-F19-G19</x:f>
@@ -1018,16 +1019,16 @@
         <x:v>Audit Records</x:v>
       </x:c>
       <x:c r="E20" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D20)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D20)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F20" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D20,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D20,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="28" t="n">
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D20,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>6</x:v>
-      </x:c>
-      <x:c r="G20" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D20,'Test Cases'!L6:L134,"Not Run")</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="H20" s="28" t="n">
         <x:f>E20-F20-G20</x:f>
@@ -1042,15 +1043,15 @@
         <x:v>Frontend Quality</x:v>
       </x:c>
       <x:c r="E21" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D21)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D21)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F21" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D21,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D21,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D21,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D21,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="H21" s="28" t="n">
@@ -1066,15 +1067,15 @@
         <x:v>Cross-Sprint Regression</x:v>
       </x:c>
       <x:c r="E22" s="28" t="n">
-        <x:f>COUNTIF('Test Cases'!C6:C134,D22)</x:f>
+        <x:f>COUNTIF('Test Cases'!$C$6:$C$134,D22)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F22" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D22,'Test Cases'!L6:L134,"Blocked")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D22,'Test Cases'!$L$6:$L$134,"Blocked")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="G22" s="28" t="n">
-        <x:f>COUNTIFS('Test Cases'!C6:C134,D22,'Test Cases'!L6:L134,"Not Run")</x:f>
+        <x:f>COUNTIFS('Test Cases'!$C$6:$C$134,D22,'Test Cases'!$L$6:$L$134,"Not Run")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H22" s="28" t="n">
@@ -1095,7 +1096,7 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="B26" t="n">
-        <x:f>COUNTIF('Test Cases'!$K$6:$K$134,A26)</x:f>
+        <x:f>COUNTIF('Test Cases'!K6:K134,A26)</x:f>
         <x:v>46</x:v>
       </x:c>
     </x:row>
@@ -1104,7 +1105,7 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="B27" t="n">
-        <x:f>COUNTIF('Test Cases'!$K$6:$K$134,A27)</x:f>
+        <x:f>COUNTIF('Test Cases'!K6:K134,A27)</x:f>
         <x:v>38</x:v>
       </x:c>
     </x:row>
@@ -1113,7 +1114,7 @@
         <x:v>Joyee</x:v>
       </x:c>
       <x:c r="B28" t="n">
-        <x:f>COUNTIF('Test Cases'!$K$6:$K$134,A28)</x:f>
+        <x:f>COUNTIF('Test Cases'!K6:K134,A28)</x:f>
         <x:v>45</x:v>
       </x:c>
     </x:row>
@@ -1132,7 +1133,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb66c4c55c93f489e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf05037759fc4425"/>
 </x:worksheet>
 </file>
 
@@ -1184,7 +1185,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="13" t="str">
-        <x:v>WBS 7.9 planning baseline. Initial execution status uses Not Run or Blocked only. Do not mark Pass or Fail until the related test is executed.</x:v>
+        <x:v>Active WBS 7.9 execution tracker. Mark Pass or Fail only after verified execution. Use Blocked only when a required dependency or environment prevents execution.</x:v>
       </x:c>
       <x:c r="B2" s="13"/>
       <x:c r="C2" s="13"/>
@@ -1436,7 +1437,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M9" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N9" s="28" t="str"/>
       <x:c r="O9" s="28" t="str"/>
@@ -1576,7 +1577,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M12" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N12" s="28" t="str"/>
       <x:c r="O12" s="28" t="str"/>
@@ -1759,16 +1760,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L16" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M16" s="28" t="str"/>
-      <x:c r="N16" s="28" t="str"/>
-      <x:c r="O16" s="28" t="str"/>
-      <x:c r="P16" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M16" s="28"/>
+      <x:c r="N16" s="28" t="str">
+        <x:v>GET /api/v1/profile/ without an access token returned HTTP 401 Unauthorized with code "not_authenticated" and message "Authentication credentials were not provided." The protected Student API rejected unauthenticated access as expected.</x:v>
+      </x:c>
+      <x:c r="O16" s="28" t="str">
+        <x:v>S4-EV-AUTH-001</x:v>
+      </x:c>
+      <x:c r="P16" s="28"/>
       <x:c r="Q16" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R16" s="28" t="str"/>
+      <x:c r="R16" s="28" t="str">
+        <x:v>Verified manually in Postman. Evidence: S4-AUTH-04_JWT_Protected_API_Without_Token_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="28" t="str">
@@ -1805,16 +1812,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L17" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M17" s="28" t="str"/>
-      <x:c r="N17" s="28" t="str"/>
-      <x:c r="O17" s="28" t="str"/>
-      <x:c r="P17" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M17" s="28"/>
+      <x:c r="N17" s="28" t="str">
+        <x:v>GET /api/v1/auth/me/ returned HTTP 200 OK for the authenticated Student. The response returned id, email, first_name, last_name, and role without exposing sensitive fields.</x:v>
+      </x:c>
+      <x:c r="O17" s="28" t="str">
+        <x:v>S4-EV-AUTH-001</x:v>
+      </x:c>
+      <x:c r="P17" s="28"/>
       <x:c r="Q17" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R17" s="28" t="str"/>
+      <x:c r="R17" s="28" t="str">
+        <x:v>Verified manually in Postman with masked Bearer token. Evidence: S4-AUTH-05_Current_User_Retrieval_After_Login_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="28" t="str">
@@ -1989,16 +2002,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L21" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M21" s="28" t="str"/>
-      <x:c r="N21" s="28" t="str"/>
-      <x:c r="O21" s="28" t="str"/>
-      <x:c r="P21" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M21" s="28"/>
+      <x:c r="N21" s="28" t="str">
+        <x:v>React was initially recognised as an existing Student Profile skill in Job Matching. After React was removed and the same job description was analysed again, the result changed from 1 of 1 matched to 0 of 1, and React moved to Not listed in your profile. React was then restored at Proficient.</x:v>
+      </x:c>
+      <x:c r="O21" s="28" t="str">
+        <x:v>S4-EV-PROFILE-001</x:v>
+      </x:c>
+      <x:c r="P21" s="28"/>
       <x:c r="Q21" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R21" s="28" t="str"/>
+      <x:c r="R21" s="28" t="str">
+        <x:v>Verified through Student Profile and Job Matching integration. Evidence: S4-PROFILE-04_Profile_Baseline_Before_Skill_Change.png; S4-PROFILE-04_Job_Matching_Baseline_React_In_Profile.png; S4-PROFILE-04_Job_Matching_After_React_Removal_PASS.png; S4-PROFILE-04_Profile_Restored_React_Proficient_Verified.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="28" t="str">
@@ -2035,16 +2054,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L22" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M22" s="28" t="str"/>
-      <x:c r="N22" s="28" t="str"/>
-      <x:c r="O22" s="28" t="str"/>
-      <x:c r="P22" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M22" s="28"/>
+      <x:c r="N22" s="28" t="str">
+        <x:v>Career Recommendations loaded successfully for the authenticated Student and returned an ordered ranked list. Software Engineer was rank #1 with an 85% Career Match, followed by ranked career matches through rank #7.</x:v>
+      </x:c>
+      <x:c r="O22" s="28" t="str">
+        <x:v>S4-EV-REC-001</x:v>
+      </x:c>
+      <x:c r="P22" s="28"/>
       <x:c r="Q22" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R22" s="28" t="str"/>
+      <x:c r="R22" s="28" t="str">
+        <x:v>Verified through Career Recommendations UI after restoring the Student Profile baseline. Evidence: S4-REC-01_Ranked_Career_Recommendations_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="28" t="str">
@@ -2127,18 +2152,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L24" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M24" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N24" s="28" t="str"/>
-      <x:c r="O24" s="28" t="str"/>
-      <x:c r="P24" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M24" s="28"/>
+      <x:c r="N24" s="28" t="str">
+        <x:v>The approved AI recommendation explanation returned successfully for the current top recommendation. After the explanation request, Career Recommendations was reloaded and Software Engineer remained rank #1 with an 85% Career Match.</x:v>
+      </x:c>
+      <x:c r="O24" s="28" t="str">
+        <x:v>S4-EV-REC-003</x:v>
+      </x:c>
+      <x:c r="P24" s="28"/>
       <x:c r="Q24" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R24" s="28" t="str"/>
+      <x:c r="R24" s="28" t="str">
+        <x:v>AI explanation returned through the approved endpoint and deterministic recommendation result remained unchanged. Evidence: S4-REC-03_AI_Recommendation_Explanation_200_OK.png; S4-REC-03_Recommendation_Rank_and_Score_Unchanged_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="28" t="str">
@@ -2175,16 +2204,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L25" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M25" s="28" t="str"/>
-      <x:c r="N25" s="28" t="str"/>
-      <x:c r="O25" s="28" t="str"/>
-      <x:c r="P25" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M25" s="28"/>
+      <x:c r="N25" s="28" t="str">
+        <x:v>The same authenticated Student profile was used for two consecutive recommendation requests. Postman compared the full recommendation arrays and confirmed the recommendation count, order, career IDs, career names, and recommendation scores repeated exactly.</x:v>
+      </x:c>
+      <x:c r="O25" s="28" t="str">
+        <x:v>S4-EV-REC-004</x:v>
+      </x:c>
+      <x:c r="P25" s="28"/>
       <x:c r="Q25" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R25" s="28" t="str"/>
+      <x:c r="R25" s="28" t="str">
+        <x:v>Postman post-response assertions passed 3/3 for full recommendation repeatability. Evidence: S4-REC-04_Recommendation_Repeatability_Run_1.png; S4-REC-04_Recommendation_Repeatability_Run_2.png; S4-REC-04_Postman_Baseline_Stored.png; S4-REC-04_Recommendation_Repeatability_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="28" t="str">
@@ -2267,18 +2302,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L27" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M27" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N27" s="28" t="str"/>
-      <x:c r="O27" s="28" t="str"/>
-      <x:c r="P27" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M27" s="28"/>
+      <x:c r="N27" s="28" t="str">
+        <x:v>A controlled AI explanation validation failure was simulated using the existing Sprint 4 backend test. The test confirmed the deterministic recommendation score, rank, evidence fields, and snapshot payload remained unchanged.</x:v>
+      </x:c>
+      <x:c r="O27" s="28" t="str">
+        <x:v>S4-EV-REC-006</x:v>
+      </x:c>
+      <x:c r="P27" s="28"/>
       <x:c r="Q27" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R27" s="28" t="str"/>
+      <x:c r="R27" s="28" t="str">
+        <x:v>Automated backend regression test passed. Evidence: S4-REC-06_AI_Explanation_Failure_Test_Setup.png; S4-REC-06_AI_Explanation_Failure_Preserves_Recommendation_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="28" t="str">
@@ -2407,16 +2446,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L30" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M30" s="28" t="str"/>
-      <x:c r="N30" s="28" t="str"/>
-      <x:c r="O30" s="28" t="str"/>
-      <x:c r="P30" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M30" s="28"/>
+      <x:c r="N30" s="28" t="str">
+        <x:v>Two consecutive Career Readiness requests were executed for Software Engineer, career_id 3, without changing the Student Profile or selected Career. Postman assertions confirmed the readiness score, requirement counts, and complete deterministic Skill Gap and readiness response repeated exactly.</x:v>
+      </x:c>
+      <x:c r="O30" s="28" t="str">
+        <x:v>S4-EV-GAP-003</x:v>
+      </x:c>
+      <x:c r="P30" s="28"/>
       <x:c r="Q30" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R30" s="28" t="str"/>
+      <x:c r="R30" s="28" t="str">
+        <x:v>Postman post-response assertions passed 4/4. Baseline readiness score was 5.54 with 0 meets, 1 below requirement, 17 missing, 18 total. Evidence: S4-GAP-03_Readiness_Baseline_Response.png; S4-GAP-03_Repeatability_Baseline_Stored.png; S4-GAP-03_Skill_Gap_Readiness_Repeatability_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="28" t="str">
@@ -2453,18 +2498,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L31" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M31" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N31" s="28" t="str"/>
-      <x:c r="O31" s="28" t="str"/>
-      <x:c r="P31" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M31" s="28"/>
+      <x:c r="N31" s="28" t="str">
+        <x:v>A controlled AI summary failure was simulated through the existing Sprint 4 backend test. The test confirmed deterministic Skill Gap and Career Readiness results were preserved during the AI failure.</x:v>
+      </x:c>
+      <x:c r="O31" s="28" t="str">
+        <x:v>S4-EV-GAP-004</x:v>
+      </x:c>
+      <x:c r="P31" s="28"/>
       <x:c r="Q31" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R31" s="28" t="str"/>
+      <x:c r="R31" s="28" t="str">
+        <x:v>Automated backend regression test passed. Evidence: S4-GAP-04_AI_Summary_Failure_Preserves_Skill_Gap_Readiness_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="28" t="str">
@@ -2501,16 +2550,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L32" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M32" s="28" t="str"/>
-      <x:c r="N32" s="28" t="str"/>
-      <x:c r="O32" s="28" t="str"/>
-      <x:c r="P32" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M32" s="28"/>
+      <x:c r="N32" s="28" t="str">
+        <x:v>The existing Sprint 4 automated test simulated an unavailable text AI provider and confirmed the deterministic Career Readiness response stayed available and unchanged.</x:v>
+      </x:c>
+      <x:c r="O32" s="28" t="str">
+        <x:v>S4-EV-GAP-005</x:v>
+      </x:c>
+      <x:c r="P32" s="28"/>
       <x:c r="Q32" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R32" s="28" t="str"/>
+      <x:c r="R32" s="28" t="str">
+        <x:v>Automated regression test passed. Evidence: S4-GAP-05_Readiness_Independent_of_Text_AI_Provider_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="28" t="str">
@@ -2961,16 +3016,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L42" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M42" s="28" t="str"/>
-      <x:c r="N42" s="28" t="str"/>
-      <x:c r="O42" s="28" t="str"/>
-      <x:c r="P42" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M42" s="28"/>
+      <x:c r="N42" s="28" t="str">
+        <x:v>A valid job description containing React, Python, Docker, and Kubernetes was submitted. GradNavi recognised all four requirements. React and Python appeared as matched Student Profile skills. Docker and Kubernetes appeared as recognised requirements absent from the Student Profile.</x:v>
+      </x:c>
+      <x:c r="O42" s="28" t="str">
+        <x:v>S4-EV-JOB-002</x:v>
+      </x:c>
+      <x:c r="P42" s="28"/>
       <x:c r="Q42" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R42" s="28" t="str"/>
+      <x:c r="R42" s="28" t="str">
+        <x:v>Verified through Job Matching UI. Evidence: S4-JOB-02_Valid_Job_Description_Matched_Missing_Requirements_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="28" t="str">
@@ -3007,16 +3068,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L43" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M43" s="28" t="str"/>
-      <x:c r="N43" s="28" t="str"/>
-      <x:c r="O43" s="28" t="str"/>
-      <x:c r="P43" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M43" s="28"/>
+      <x:c r="N43" s="28" t="str">
+        <x:v>The Job Matching page was opened with an empty job-description field. The field showed 0 / 20,000 characters and the Analyze Job action was disabled, preventing submission of blank input.</x:v>
+      </x:c>
+      <x:c r="O43" s="28" t="str">
+        <x:v>S4-EV-JOB-003</x:v>
+      </x:c>
+      <x:c r="P43" s="28"/>
       <x:c r="Q43" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R43" s="28" t="str"/>
+      <x:c r="R43" s="28" t="str">
+        <x:v>Frontend validation verified manually. Evidence: S4-JOB-03_Blank_Job_Description_Validation_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="28" t="str">
@@ -3053,16 +3120,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L44" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M44" s="28" t="str"/>
-      <x:c r="N44" s="28" t="str"/>
-      <x:c r="O44" s="28" t="str"/>
-      <x:c r="P44" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M44" s="28"/>
+      <x:c r="N44" s="28" t="str">
+        <x:v>A 20,001-character job description exceeded the approved 20,000-character limit. The interface displayed 1 over limit and disabled Analyze Job, preventing submission.</x:v>
+      </x:c>
+      <x:c r="O44" s="28" t="str">
+        <x:v>S4-EV-JOB-004</x:v>
+      </x:c>
+      <x:c r="P44" s="28"/>
       <x:c r="Q44" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R44" s="28" t="str"/>
+      <x:c r="R44" s="28" t="str">
+        <x:v>Frontend oversized-input validation verified manually. Evidence: S4-JOB-04_Oversized_Job_Description_Validation_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="28" t="str">
@@ -3191,16 +3264,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L47" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M47" s="28" t="str"/>
-      <x:c r="N47" s="28" t="str"/>
-      <x:c r="O47" s="28" t="str"/>
-      <x:c r="P47" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M47" s="28"/>
+      <x:c r="N47" s="28" t="str">
+        <x:v>A job description containing the canonical Skill name React was submitted. GradNavi recognised React, resolved the requirement directly to the canonical React Skill, identified the match source as Canonical match, and matched it against the authenticated Student Profile.</x:v>
+      </x:c>
+      <x:c r="O47" s="28" t="str">
+        <x:v>S4-EV-JOB-007</x:v>
+      </x:c>
+      <x:c r="P47" s="28"/>
       <x:c r="Q47" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R47" s="28" t="str"/>
+      <x:c r="R47" s="28" t="str">
+        <x:v>Verified through Job Matching UI. Evidence: S4-JOB-07_Canonical_Skill_Matching_React_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="28" t="str">
@@ -3237,16 +3316,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L48" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M48" s="28" t="str"/>
-      <x:c r="N48" s="28" t="str"/>
-      <x:c r="O48" s="28" t="str"/>
-      <x:c r="P48" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M48" s="28"/>
+      <x:c r="N48" s="28" t="str">
+        <x:v>The existing Sprint 4 automated test submitted the approved SkillAlias "Py". GradNavi resolved the alias to the canonical Python Skill and identified the match source as alias.</x:v>
+      </x:c>
+      <x:c r="O48" s="28" t="str">
+        <x:v>S4-EV-JOB-008</x:v>
+      </x:c>
+      <x:c r="P48" s="28"/>
       <x:c r="Q48" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R48" s="28" t="str"/>
+      <x:c r="R48" s="28" t="str">
+        <x:v>Automated backend test passed. Evidence: S4-JOB-08_Skill_Alias_Matching_Py_to_Python_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="28" t="str">
@@ -3283,16 +3368,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L49" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M49" s="28" t="str"/>
-      <x:c r="N49" s="28" t="str"/>
-      <x:c r="O49" s="28" t="str"/>
-      <x:c r="P49" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M49" s="28"/>
+      <x:c r="N49" s="28" t="str">
+        <x:v>The existing Sprint 4 automated test submitted unsupported generic terms including testing, APIs, software development, problem solving, and communication. GradNavi returned no guessed Skill requirements.</x:v>
+      </x:c>
+      <x:c r="O49" s="28" t="str">
+        <x:v>S4-EV-JOB-009</x:v>
+      </x:c>
+      <x:c r="P49" s="28"/>
       <x:c r="Q49" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R49" s="28" t="str"/>
+      <x:c r="R49" s="28" t="str">
+        <x:v>Automated backend test passed. Evidence: S4-JOB-09_Unsupported_Synonym_Guessing_Not_Guessed_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="28" t="str">
@@ -3329,16 +3420,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L50" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M50" s="28" t="str"/>
-      <x:c r="N50" s="28" t="str"/>
-      <x:c r="O50" s="28" t="str"/>
-      <x:c r="P50" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M50" s="28"/>
+      <x:c r="N50" s="28" t="str">
+        <x:v>The existing Sprint 4 automated test used generic design wording without approved requirement context. GradNavi did not incorrectly resolve the wording to the canonical Design concept.</x:v>
+      </x:c>
+      <x:c r="O50" s="28" t="str">
+        <x:v>S4-EV-JOB-010</x:v>
+      </x:c>
+      <x:c r="P50" s="28"/>
       <x:c r="Q50" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R50" s="28" t="str"/>
+      <x:c r="R50" s="28" t="str">
+        <x:v>Automated backend test passed. Evidence: S4-JOB-10_Generic_Design_False_Positive_Avoided_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="28" t="str">
@@ -3375,16 +3472,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L51" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M51" s="28" t="str"/>
-      <x:c r="N51" s="28" t="str"/>
-      <x:c r="O51" s="28" t="str"/>
-      <x:c r="P51" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M51" s="28"/>
+      <x:c r="N51" s="28" t="str">
+        <x:v>The Job Matching API response contract test passed. The approved response contains structured matched and missing requirement data and does not expose a hiring probability or employment suitability score. The Job Matching UI also states the result is not an employment suitability score.</x:v>
+      </x:c>
+      <x:c r="O51" s="28" t="str">
+        <x:v>S4-EV-JOB-011</x:v>
+      </x:c>
+      <x:c r="P51" s="28"/>
       <x:c r="Q51" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R51" s="28" t="str"/>
+      <x:c r="R51" s="28" t="str">
+        <x:v>API contract and existing UI evidence verified. Evidence: S4-JOB-11_No_Suitability_Score_API_Contract_PASS.png; S4-JOB-02_Valid_Job_Description_Matched_Missing_Requirements_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="28" t="str">
@@ -3421,16 +3524,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L52" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M52" s="28" t="str"/>
-      <x:c r="N52" s="28" t="str"/>
-      <x:c r="O52" s="28" t="str"/>
-      <x:c r="P52" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M52" s="28"/>
+      <x:c r="N52" s="28" t="str">
+        <x:v>The Sprint 4 API test submitted a valid job description with an unsupported student_profile_id ownership field. The backend rejected the unsupported field with validation rather than accepting a client ownership override.</x:v>
+      </x:c>
+      <x:c r="O52" s="28" t="str">
+        <x:v>S4-EV-JOB-012</x:v>
+      </x:c>
+      <x:c r="P52" s="28"/>
       <x:c r="Q52" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R52" s="28" t="str"/>
+      <x:c r="R52" s="28" t="str">
+        <x:v>Automated backend ownership-contract test passed. Evidence: S4-JOB-12_Reject_Client_Ownership_Override_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="28" t="str">
@@ -3467,16 +3576,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L53" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M53" s="28" t="str"/>
-      <x:c r="N53" s="28" t="str"/>
-      <x:c r="O53" s="28" t="str"/>
-      <x:c r="P53" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M53" s="28"/>
+      <x:c r="N53" s="28" t="str">
+        <x:v>Multiple Job Matching operations were completed and the Student Profile was reloaded. The profile retained the original six Skills, three Career Goals with Software Engineer as Primary, and four Interests. Job Matching did not mutate the Student Profile.</x:v>
+      </x:c>
+      <x:c r="O53" s="28" t="str">
+        <x:v>S4-EV-JOB-013</x:v>
+      </x:c>
+      <x:c r="P53" s="28"/>
       <x:c r="Q53" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R53" s="28" t="str"/>
+      <x:c r="R53" s="28" t="str">
+        <x:v>Evidence: S4-JOB-13_Job_Matching_Does_Not_Mutate_Profile_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="28" t="str">
@@ -3789,18 +3904,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L60" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M60" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N60" s="28" t="str"/>
-      <x:c r="O60" s="28" t="str"/>
-      <x:c r="P60" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M60" s="28"/>
+      <x:c r="N60" s="28" t="str">
+        <x:v>The Sprint 4 Resume API automated test simulated an unavailable AI provider. The API returned the approved HTTP 503 external-service-unavailable response, and Resume generation did not proceed.</x:v>
+      </x:c>
+      <x:c r="O60" s="28" t="str">
+        <x:v>S4-EV-RESUME-005</x:v>
+      </x:c>
+      <x:c r="P60" s="28"/>
       <x:c r="Q60" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R60" s="28" t="str"/>
+      <x:c r="R60" s="28" t="str">
+        <x:v>Automated backend test passed. Evidence: S4-RESUME-05_Resume_Provider_Failure_Controlled_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="28" t="str">
@@ -3837,18 +3956,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L61" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M61" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N61" s="28" t="str"/>
-      <x:c r="O61" s="28" t="str"/>
-      <x:c r="P61" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M61" s="28"/>
+      <x:c r="N61" s="28" t="str">
+        <x:v>The Sprint 4 Resume API automated test simulated an AI response-validation failure. The API returned the approved sanitized HTTP 503 external-service-unavailable response and did not expose sensitive provider details, submitted job-description content, or internal OpenAI validation information.</x:v>
+      </x:c>
+      <x:c r="O61" s="28" t="str">
+        <x:v>S4-EV-RESUME-006</x:v>
+      </x:c>
+      <x:c r="P61" s="28"/>
       <x:c r="Q61" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R61" s="28" t="str"/>
+      <x:c r="R61" s="28" t="str">
+        <x:v>Automated backend test passed. Evidence: S4-RESUME-06_Invalid_AI_Response_Rejected_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="28" t="str">
@@ -4161,18 +4284,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L68" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M68" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N68" s="28" t="str"/>
-      <x:c r="O68" s="28" t="str"/>
-      <x:c r="P68" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M68" s="28"/>
+      <x:c r="N68" s="28" t="str">
+        <x:v>The Sprint 4 Cover Letter API automated test simulated an unavailable AI provider. The API returned the approved controlled service-unavailable response and prevented Cover Letter generation.</x:v>
+      </x:c>
+      <x:c r="O68" s="28" t="str">
+        <x:v>S4-EV-COVER-006</x:v>
+      </x:c>
+      <x:c r="P68" s="28"/>
       <x:c r="Q68" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R68" s="28" t="str"/>
+      <x:c r="R68" s="28" t="str">
+        <x:v>Automated backend test passed. Evidence: S4-COVER-06_Cover_Letter_Provider_Failure_Controlled_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="28" t="str">
@@ -4301,16 +4428,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L71" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M71" s="28" t="str"/>
-      <x:c r="N71" s="28" t="str"/>
-      <x:c r="O71" s="28" t="str"/>
-      <x:c r="P71" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M71" s="28"/>
+      <x:c r="N71" s="28" t="str">
+        <x:v>An authenticated request for five Software Engineer interview questions returned HTTP 200 OK. GradNavi returned a structured question set containing five role-relevant questions with focus areas based on the supplied job description.</x:v>
+      </x:c>
+      <x:c r="O71" s="28" t="str">
+        <x:v>S4-EV-INT-002</x:v>
+      </x:c>
+      <x:c r="P71" s="28"/>
       <x:c r="Q71" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R71" s="28" t="str"/>
+      <x:c r="R71" s="28" t="str">
+        <x:v>Verified manually in Postman. Evidence: S4-INT-02_Generate_Valid_Interview_Questions_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="28" t="str">
@@ -4347,16 +4480,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L72" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M72" s="28" t="str"/>
-      <x:c r="N72" s="28" t="str"/>
-      <x:c r="O72" s="28" t="str"/>
-      <x:c r="P72" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M72" s="28"/>
+      <x:c r="N72" s="28" t="str">
+        <x:v>An authenticated Interview Questions request with question_count set to 0 returned HTTP 400 Bad Request. GradNavi returned the controlled validation_error response and identified question_count as requiring a value of at least 1.</x:v>
+      </x:c>
+      <x:c r="O72" s="28" t="str">
+        <x:v>S4-EV-INT-003</x:v>
+      </x:c>
+      <x:c r="P72" s="28"/>
       <x:c r="Q72" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R72" s="28" t="str"/>
+      <x:c r="R72" s="28" t="str">
+        <x:v>Verified manually in Postman. Evidence: S4-INT-03_Reject_Question_Count_Below_Range_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="28" t="str">
@@ -4393,16 +4532,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L73" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M73" s="28" t="str"/>
-      <x:c r="N73" s="28" t="str"/>
-      <x:c r="O73" s="28" t="str"/>
-      <x:c r="P73" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M73" s="28"/>
+      <x:c r="N73" s="28" t="str">
+        <x:v>An authenticated Interview Questions request with question_count set to 11 returned HTTP 400 Bad Request. GradNavi returned the controlled validation_error response and identified question_count as exceeding the maximum value of 10.</x:v>
+      </x:c>
+      <x:c r="O73" s="28" t="str">
+        <x:v>S4-EV-INT-004</x:v>
+      </x:c>
+      <x:c r="P73" s="28"/>
       <x:c r="Q73" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R73" s="28" t="str"/>
+      <x:c r="R73" s="28" t="str">
+        <x:v>Verified manually in Postman. Evidence: S4-INT-04_Reject_Question_Count_Above_Range_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="28" t="str">
@@ -4531,16 +4676,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L76" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M76" s="28" t="str"/>
-      <x:c r="N76" s="28" t="str"/>
-      <x:c r="O76" s="28" t="str"/>
-      <x:c r="P76" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M76" s="28"/>
+      <x:c r="N76" s="28" t="str">
+        <x:v>An authenticated Interview Feedback request returned HTTP 200 OK. GradNavi returned structured strengths, improvements, and a suggested response based on the submitted interview answer.</x:v>
+      </x:c>
+      <x:c r="O76" s="28" t="str">
+        <x:v>S4-EV-INT-007</x:v>
+      </x:c>
+      <x:c r="P76" s="28"/>
       <x:c r="Q76" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R76" s="28" t="str"/>
+      <x:c r="R76" s="28" t="str">
+        <x:v>Verified manually in Postman. Evidence: S4-INT-07_Generate_Structured_Interview_Feedback_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="28" t="str">
@@ -4577,18 +4728,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L77" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M77" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N77" s="28" t="str"/>
-      <x:c r="O77" s="28" t="str"/>
-      <x:c r="P77" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M77" s="28"/>
+      <x:c r="N77" s="28" t="str">
+        <x:v>The Sprint 4 Interview Questions automated test supplied a semantically invalid AI response with mismatched focus areas. GradNavi rejected the response through the controlled HTTP 502 validation path and prevented sensitive internal details from appearing in the response.</x:v>
+      </x:c>
+      <x:c r="O77" s="28" t="str">
+        <x:v>S4-EV-INT-008</x:v>
+      </x:c>
+      <x:c r="P77" s="28"/>
       <x:c r="Q77" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R77" s="28" t="str"/>
+      <x:c r="R77" s="28" t="str">
+        <x:v>Automated backend test passed. Evidence: S4-INT-08_Reject_Semantically_Invalid_Focus_Areas_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="28" t="str">
@@ -4625,16 +4780,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L78" s="28" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="M78" s="28" t="str"/>
-      <x:c r="N78" s="28" t="str"/>
-      <x:c r="O78" s="28" t="str"/>
-      <x:c r="P78" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M78" s="28"/>
+      <x:c r="N78" s="28" t="str">
+        <x:v>The Sprint 4 Interview Questions and Interview Feedback response-contract tests both passed. Neither response includes hiring_probability or pass_fail fields, while the approved structured output fields remain available.</x:v>
+      </x:c>
+      <x:c r="O78" s="28" t="str">
+        <x:v>S4-EV-INT-009</x:v>
+      </x:c>
+      <x:c r="P78" s="28"/>
       <x:c r="Q78" s="28" t="str">
         <x:v>Hybrid</x:v>
       </x:c>
-      <x:c r="R78" s="28" t="str"/>
+      <x:c r="R78" s="28" t="str">
+        <x:v>Two automated backend contract tests passed. Evidence: S4-INT-09_Exclude_Hiring_Probability_Pass_Fail_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="28" t="str">
@@ -4671,18 +4832,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L79" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M79" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N79" s="28" t="str"/>
-      <x:c r="O79" s="28" t="str"/>
-      <x:c r="P79" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M79" s="28"/>
+      <x:c r="N79" s="28" t="str">
+        <x:v>The Sprint 4 OpenAI text-provider test supplied a completed provider response with valid structured output. GradNavi accepted the response, validated the structured content, and returned the approved output successfully.</x:v>
+      </x:c>
+      <x:c r="O79" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-001</x:v>
+      </x:c>
+      <x:c r="P79" s="28"/>
       <x:c r="Q79" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R79" s="28" t="str"/>
+      <x:c r="R79" s="28" t="str">
+        <x:v>Automated provider-validation test passed. Evidence: S4-AI-01_Accept_Completed_AI_Response_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="28" t="str">
@@ -4719,18 +4884,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L80" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M80" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N80" s="28" t="str"/>
-      <x:c r="O80" s="28" t="str"/>
-      <x:c r="P80" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M80" s="28"/>
+      <x:c r="N80" s="28" t="str">
+        <x:v>The OpenAI text-provider automated test supplied an incomplete AI response. GradNavi rejected the response through the approved validation layer.</x:v>
+      </x:c>
+      <x:c r="O80" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-002</x:v>
+      </x:c>
+      <x:c r="P80" s="28"/>
       <x:c r="Q80" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R80" s="28" t="str"/>
+      <x:c r="R80" s="28" t="str">
+        <x:v>Automated provider-validation test passed. Evidence: S4-AI-02_Reject_Incomplete_AI_Response_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="28" t="str">
@@ -4767,18 +4936,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L81" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M81" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N81" s="28" t="str"/>
-      <x:c r="O81" s="28" t="str"/>
-      <x:c r="P81" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M81" s="28"/>
+      <x:c r="N81" s="28" t="str">
+        <x:v>The OpenAI text-provider validation test supplied a failed response state. GradNavi rejected the response instead of accepting AI output.</x:v>
+      </x:c>
+      <x:c r="O81" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-003</x:v>
+      </x:c>
+      <x:c r="P81" s="28"/>
       <x:c r="Q81" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R81" s="28" t="str"/>
+      <x:c r="R81" s="28" t="str">
+        <x:v>Covered by shared non-completed-state automated test. Evidence: S4-AI-03-05_Reject_Non_Completed_AI_Response_States_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="28" t="str">
@@ -4815,18 +4988,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L82" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M82" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N82" s="28" t="str"/>
-      <x:c r="O82" s="28" t="str"/>
-      <x:c r="P82" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M82" s="28"/>
+      <x:c r="N82" s="28" t="str">
+        <x:v>The OpenAI text-provider validation test supplied a cancelled response state. GradNavi rejected the response instead of accepting AI output.</x:v>
+      </x:c>
+      <x:c r="O82" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-004</x:v>
+      </x:c>
+      <x:c r="P82" s="28"/>
       <x:c r="Q82" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R82" s="28" t="str"/>
+      <x:c r="R82" s="28" t="str">
+        <x:v>Covered by shared non-completed-state automated test. Evidence: S4-AI-03-05_Reject_Non_Completed_AI_Response_States_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="28" t="str">
@@ -4863,18 +5040,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L83" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M83" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N83" s="28" t="str"/>
-      <x:c r="O83" s="28" t="str"/>
-      <x:c r="P83" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M83" s="28"/>
+      <x:c r="N83" s="28" t="str">
+        <x:v>The OpenAI text-provider validation test supplied queued and in_progress response states. GradNavi rejected both non-completed states.</x:v>
+      </x:c>
+      <x:c r="O83" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-005</x:v>
+      </x:c>
+      <x:c r="P83" s="28"/>
       <x:c r="Q83" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R83" s="28" t="str"/>
+      <x:c r="R83" s="28" t="str">
+        <x:v>Covered by shared non-completed-state automated test. Evidence: S4-AI-03-05_Reject_Non_Completed_AI_Response_States_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="28" t="str">
@@ -4911,18 +5092,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L84" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M84" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N84" s="28" t="str"/>
-      <x:c r="O84" s="28" t="str"/>
-      <x:c r="P84" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M84" s="28"/>
+      <x:c r="N84" s="28" t="str">
+        <x:v>The OpenAI text-provider automated test supplied an AI response without a response status. GradNavi rejected the response through the approved validation layer.</x:v>
+      </x:c>
+      <x:c r="O84" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-006</x:v>
+      </x:c>
+      <x:c r="P84" s="28"/>
       <x:c r="Q84" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R84" s="28" t="str"/>
+      <x:c r="R84" s="28" t="str">
+        <x:v>Automated provider-validation test passed. Evidence: S4-AI-06_Reject_Missing_AI_Response_Status_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="28" t="str">
@@ -4959,18 +5144,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L85" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M85" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N85" s="28" t="str"/>
-      <x:c r="O85" s="28" t="str"/>
-      <x:c r="P85" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M85" s="28"/>
+      <x:c r="N85" s="28" t="str">
+        <x:v>The OpenAI text-provider automated test supplied a completed AI response with empty output. GradNavi rejected the response through the approved structured-output validation process.</x:v>
+      </x:c>
+      <x:c r="O85" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-007</x:v>
+      </x:c>
+      <x:c r="P85" s="28"/>
       <x:c r="Q85" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R85" s="28" t="str"/>
+      <x:c r="R85" s="28" t="str">
+        <x:v>Automated provider-validation test passed. Evidence: S4-AI-07_Reject_Empty_AI_Output_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="28" t="str">
@@ -5007,18 +5196,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L86" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M86" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N86" s="28" t="str"/>
-      <x:c r="O86" s="28" t="str"/>
-      <x:c r="P86" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M86" s="28"/>
+      <x:c r="N86" s="28" t="str">
+        <x:v>The OpenAI text-provider automated test supplied a completed AI response containing malformed JSON. GradNavi rejected the malformed structured output through the approved AI response-validation process.</x:v>
+      </x:c>
+      <x:c r="O86" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-008</x:v>
+      </x:c>
+      <x:c r="P86" s="28"/>
       <x:c r="Q86" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R86" s="28" t="str"/>
+      <x:c r="R86" s="28" t="str">
+        <x:v>Automated provider-validation test passed. Evidence: S4-AI-08_Reject_Malformed_AI_JSON_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="28" t="str">
@@ -5055,18 +5248,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L87" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M87" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N87" s="28" t="str"/>
-      <x:c r="O87" s="28" t="str"/>
-      <x:c r="P87" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M87" s="28"/>
+      <x:c r="N87" s="28" t="str">
+        <x:v>The OpenAI text-provider automated test simulated a provider timeout. GradNavi translated the failure into the approved application-level error and did not expose provider-specific timeout details.</x:v>
+      </x:c>
+      <x:c r="O87" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-009</x:v>
+      </x:c>
+      <x:c r="P87" s="28"/>
       <x:c r="Q87" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R87" s="28" t="str"/>
+      <x:c r="R87" s="28" t="str">
+        <x:v>Automated provider-failure test passed. Evidence: S4-AI-09_Translate_Provider_Timeout_Safely_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="28" t="str">
@@ -5103,18 +5300,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L88" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M88" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N88" s="28" t="str"/>
-      <x:c r="O88" s="28" t="str"/>
-      <x:c r="P88" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M88" s="28"/>
+      <x:c r="N88" s="28" t="str">
+        <x:v>The OpenAI text-provider automated test simulated a provider connection failure. GradNavi sanitized the failure and translated it into the approved application-level AI service error without exposing provider-specific details.</x:v>
+      </x:c>
+      <x:c r="O88" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-010</x:v>
+      </x:c>
+      <x:c r="P88" s="28"/>
       <x:c r="Q88" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R88" s="28" t="str"/>
+      <x:c r="R88" s="28" t="str">
+        <x:v>Automated provider-failure test passed. Evidence: S4-AI-10_Translate_Connection_Failure_Safely_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="28" t="str">
@@ -5151,18 +5352,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L89" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M89" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N89" s="28" t="str"/>
-      <x:c r="O89" s="28" t="str"/>
-      <x:c r="P89" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M89" s="28"/>
+      <x:c r="N89" s="28" t="str">
+        <x:v>The Sprint 4 OpenAI text-provider tests simulated a provider rate-limit failure and a provider HTTP status failure. GradNavi sanitized both failures and prevented provider-specific details from being exposed.</x:v>
+      </x:c>
+      <x:c r="O89" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-011</x:v>
+      </x:c>
+      <x:c r="P89" s="28"/>
       <x:c r="Q89" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R89" s="28" t="str"/>
+      <x:c r="R89" s="28" t="str">
+        <x:v>Two automated provider-failure tests passed. Evidence: S4-AI-11_Translate_Rate_Limit_HTTP_Failure_Safely_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="28" t="str">
@@ -5199,18 +5404,22 @@
         <x:v>Jerald</x:v>
       </x:c>
       <x:c r="L90" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M90" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
-      </x:c>
-      <x:c r="N90" s="28" t="str"/>
-      <x:c r="O90" s="28" t="str"/>
-      <x:c r="P90" s="28" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M90" s="28"/>
+      <x:c r="N90" s="28" t="str">
+        <x:v>The Sprint 4 regression tests confirmed that AI failure does not change deterministic Career Recommendation scoring, Skill Gap results, Career Readiness results, or Job Matching output. All three automated tests passed.</x:v>
+      </x:c>
+      <x:c r="O90" s="28" t="str">
+        <x:v>S4-EV-AI-CASE-012</x:v>
+      </x:c>
+      <x:c r="P90" s="28"/>
       <x:c r="Q90" s="28" t="str">
         <x:v>Automated</x:v>
       </x:c>
-      <x:c r="R90" s="28" t="str"/>
+      <x:c r="R90" s="28" t="str">
+        <x:v>Three deterministic-protection tests passed. Evidence: S4-AI-12_Protect_Deterministic_Results_During_AI_Failure_PASS.png</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="28" t="str">
@@ -5247,11 +5456,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L91" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M91" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M91" s="28"/>
       <x:c r="N91" s="28" t="str"/>
       <x:c r="O91" s="28" t="str"/>
       <x:c r="P91" s="28" t="str"/>
@@ -5295,11 +5502,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L92" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M92" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M92" s="28"/>
       <x:c r="N92" s="28" t="str"/>
       <x:c r="O92" s="28" t="str"/>
       <x:c r="P92" s="28" t="str"/>
@@ -5343,11 +5548,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L93" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M93" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M93" s="28"/>
       <x:c r="N93" s="28" t="str"/>
       <x:c r="O93" s="28" t="str"/>
       <x:c r="P93" s="28" t="str"/>
@@ -5391,11 +5594,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L94" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M94" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M94" s="28"/>
       <x:c r="N94" s="28" t="str"/>
       <x:c r="O94" s="28" t="str"/>
       <x:c r="P94" s="28" t="str"/>
@@ -5439,11 +5640,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L95" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M95" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M95" s="28"/>
       <x:c r="N95" s="28" t="str"/>
       <x:c r="O95" s="28" t="str"/>
       <x:c r="P95" s="28" t="str"/>
@@ -5487,11 +5686,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L96" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M96" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M96" s="28"/>
       <x:c r="N96" s="28" t="str"/>
       <x:c r="O96" s="28" t="str"/>
       <x:c r="P96" s="28" t="str"/>
@@ -5535,11 +5732,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L97" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M97" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M97" s="28"/>
       <x:c r="N97" s="28" t="str"/>
       <x:c r="O97" s="28" t="str"/>
       <x:c r="P97" s="28" t="str"/>
@@ -5583,11 +5778,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L98" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M98" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M98" s="28"/>
       <x:c r="N98" s="28" t="str"/>
       <x:c r="O98" s="28" t="str"/>
       <x:c r="P98" s="28" t="str"/>
@@ -5631,11 +5824,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L99" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M99" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M99" s="28"/>
       <x:c r="N99" s="28" t="str"/>
       <x:c r="O99" s="28" t="str"/>
       <x:c r="P99" s="28" t="str"/>
@@ -5679,11 +5870,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L100" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M100" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M100" s="28"/>
       <x:c r="N100" s="28" t="str"/>
       <x:c r="O100" s="28" t="str"/>
       <x:c r="P100" s="28" t="str"/>
@@ -5730,7 +5919,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M101" s="28" t="str">
-        <x:v>WBS 7.7 and WBS 7.6</x:v>
+        <x:v>WBS 7.7</x:v>
       </x:c>
       <x:c r="N101" s="28" t="str"/>
       <x:c r="O101" s="28" t="str"/>
@@ -5778,7 +5967,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M102" s="28" t="str">
-        <x:v>WBS 7.7 and WBS 7.6</x:v>
+        <x:v>WBS 7.7</x:v>
       </x:c>
       <x:c r="N102" s="28" t="str"/>
       <x:c r="O102" s="28" t="str"/>
@@ -5826,7 +6015,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M103" s="28" t="str">
-        <x:v>WBS 7.7 and WBS 7.6</x:v>
+        <x:v>WBS 7.7</x:v>
       </x:c>
       <x:c r="N103" s="28" t="str"/>
       <x:c r="O103" s="28" t="str"/>
@@ -5874,7 +6063,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M104" s="28" t="str">
-        <x:v>WBS 7.7 and WBS 7.6</x:v>
+        <x:v>WBS 7.7</x:v>
       </x:c>
       <x:c r="N104" s="28" t="str"/>
       <x:c r="O104" s="28" t="str"/>
@@ -5922,7 +6111,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M105" s="28" t="str">
-        <x:v>WBS 7.7 and WBS 7.6</x:v>
+        <x:v>WBS 7.7</x:v>
       </x:c>
       <x:c r="N105" s="28" t="str"/>
       <x:c r="O105" s="28" t="str"/>
@@ -5970,7 +6159,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M106" s="28" t="str">
-        <x:v>WBS 7.7 and WBS 7.6</x:v>
+        <x:v>WBS 7.7</x:v>
       </x:c>
       <x:c r="N106" s="28" t="str"/>
       <x:c r="O106" s="28" t="str"/>
@@ -6018,7 +6207,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M107" s="28" t="str">
-        <x:v>WBS 7.7 and WBS 7.6</x:v>
+        <x:v>WBS 7.7</x:v>
       </x:c>
       <x:c r="N107" s="28" t="str"/>
       <x:c r="O107" s="28" t="str"/>
@@ -6066,7 +6255,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M108" s="28" t="str">
-        <x:v>WBS 7.7 and WBS 7.6</x:v>
+        <x:v>WBS 7.7</x:v>
       </x:c>
       <x:c r="N108" s="28" t="str"/>
       <x:c r="O108" s="28" t="str"/>
@@ -6111,11 +6300,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L109" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M109" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M109" s="28"/>
       <x:c r="N109" s="28" t="str"/>
       <x:c r="O109" s="28" t="str"/>
       <x:c r="P109" s="28" t="str"/>
@@ -6159,11 +6346,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L110" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M110" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M110" s="28"/>
       <x:c r="N110" s="28" t="str"/>
       <x:c r="O110" s="28" t="str"/>
       <x:c r="P110" s="28" t="str"/>
@@ -6207,11 +6392,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L111" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M111" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M111" s="28"/>
       <x:c r="N111" s="28" t="str"/>
       <x:c r="O111" s="28" t="str"/>
       <x:c r="P111" s="28" t="str"/>
@@ -6255,11 +6438,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L112" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M112" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M112" s="28"/>
       <x:c r="N112" s="28" t="str"/>
       <x:c r="O112" s="28" t="str"/>
       <x:c r="P112" s="28" t="str"/>
@@ -6303,11 +6484,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L113" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M113" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M113" s="28"/>
       <x:c r="N113" s="28" t="str"/>
       <x:c r="O113" s="28" t="str"/>
       <x:c r="P113" s="28" t="str"/>
@@ -6351,11 +6530,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L114" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M114" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M114" s="28"/>
       <x:c r="N114" s="28" t="str"/>
       <x:c r="O114" s="28" t="str"/>
       <x:c r="P114" s="28" t="str"/>
@@ -6399,11 +6576,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L115" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M115" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M115" s="28"/>
       <x:c r="N115" s="28" t="str"/>
       <x:c r="O115" s="28" t="str"/>
       <x:c r="P115" s="28" t="str"/>
@@ -6447,11 +6622,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L116" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M116" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M116" s="28"/>
       <x:c r="N116" s="28" t="str"/>
       <x:c r="O116" s="28" t="str"/>
       <x:c r="P116" s="28" t="str"/>
@@ -6495,11 +6668,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L117" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M117" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M117" s="28"/>
       <x:c r="N117" s="28" t="str"/>
       <x:c r="O117" s="28" t="str"/>
       <x:c r="P117" s="28" t="str"/>
@@ -6543,11 +6714,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L118" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M118" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M118" s="28"/>
       <x:c r="N118" s="28" t="str"/>
       <x:c r="O118" s="28" t="str"/>
       <x:c r="P118" s="28" t="str"/>
@@ -6591,11 +6760,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L119" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M119" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M119" s="28"/>
       <x:c r="N119" s="28" t="str"/>
       <x:c r="O119" s="28" t="str"/>
       <x:c r="P119" s="28" t="str"/>
@@ -6639,11 +6806,9 @@
         <x:v>MD</x:v>
       </x:c>
       <x:c r="L120" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="M120" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
-      </x:c>
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="M120" s="28"/>
       <x:c r="N120" s="28" t="str"/>
       <x:c r="O120" s="28" t="str"/>
       <x:c r="P120" s="28" t="str"/>
@@ -6922,7 +7087,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M126" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N126" s="28" t="str"/>
       <x:c r="O126" s="28" t="str"/>
@@ -6970,7 +7135,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M127" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N127" s="28" t="str"/>
       <x:c r="O127" s="28" t="str"/>
@@ -7018,7 +7183,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M128" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N128" s="28" t="str"/>
       <x:c r="O128" s="28" t="str"/>
@@ -7066,7 +7231,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M129" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N129" s="28" t="str"/>
       <x:c r="O129" s="28" t="str"/>
@@ -7114,7 +7279,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M130" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N130" s="28" t="str"/>
       <x:c r="O130" s="28" t="str"/>
@@ -7162,7 +7327,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M131" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N131" s="28" t="str"/>
       <x:c r="O131" s="28" t="str"/>
@@ -7210,7 +7375,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M132" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N132" s="28" t="str"/>
       <x:c r="O132" s="28" t="str"/>
@@ -7258,7 +7423,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M133" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N133" s="28" t="str"/>
       <x:c r="O133" s="28" t="str"/>
@@ -7306,7 +7471,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M134" s="28" t="str">
-        <x:v>WBS 7.4, 7.6, 7.7, 7.8 integration gate</x:v>
+        <x:v>WBS 7.7 integration gate</x:v>
       </x:c>
       <x:c r="N134" s="28" t="str"/>
       <x:c r="O134" s="28" t="str"/>
@@ -7357,7 +7522,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196476165ba04ed0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97499131a937459d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7489,10 +7654,14 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="H7" s="28" t="str">
-        <x:v>Planned</x:v>
-      </x:c>
-      <x:c r="I7" s="28" t="str"/>
-      <x:c r="J7" s="28" t="str"/>
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="I7" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J7" s="28" t="str">
+        <x:v>Detailed captured evidence entries for completed Job Matching tests are listed below.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="28" t="str">
@@ -7514,14 +7683,16 @@
         <x:v>docs/testing/evidence/sprint-4/</x:v>
       </x:c>
       <x:c r="G8" s="28" t="str">
-        <x:v>All Members</x:v>
+        <x:v>Jerald</x:v>
       </x:c>
       <x:c r="H8" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I8" s="28" t="str"/>
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I8" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
       <x:c r="J8" s="28" t="str">
-        <x:v>WBS 7.4</x:v>
+        <x:v>All S4-AI-01 to S4-AI-12 cases assigned to Jerald have been executed and passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7547,10 +7718,14 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="H9" s="28" t="str">
-        <x:v>Planned</x:v>
-      </x:c>
-      <x:c r="I9" s="28" t="str"/>
-      <x:c r="J9" s="28" t="str"/>
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="I9" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J9" s="28" t="str">
+        <x:v>Jerald-owned Resume and Cover Letter failure-path tests are captured. Other assigned document tests remain Not Run.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="28" t="str">
@@ -7575,10 +7750,14 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="H10" s="28" t="str">
-        <x:v>Planned</x:v>
-      </x:c>
-      <x:c r="I10" s="28" t="str"/>
-      <x:c r="J10" s="28" t="str"/>
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="I10" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J10" s="28" t="str">
+        <x:v>Jerald-owned Interview API and validation tests are captured. Joyee-owned UI tests remain Not Run.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="28" t="str">
@@ -7603,11 +7782,11 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="H11" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I11" s="28" t="str"/>
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I11" s="28"/>
       <x:c r="J11" s="28" t="str">
-        <x:v>WBS 7.6</x:v>
+        <x:v>WBS 7.6 is integrated. Admin API tests are ready for execution.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7635,9 +7814,9 @@
       <x:c r="H12" s="28" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="I12" s="28" t="str"/>
+      <x:c r="I12" s="28"/>
       <x:c r="J12" s="28" t="str">
-        <x:v>WBS 7.7</x:v>
+        <x:v>WBS 7.7 remains in progress. Admin Dashboard UI evidence stays blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -7663,11 +7842,11 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="H13" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I13" s="28" t="str"/>
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I13" s="28"/>
       <x:c r="J13" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
+        <x:v>WBS 7.8 is integrated. Role Permission tests are ready for execution.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -7693,11 +7872,11 @@
         <x:v>All Members</x:v>
       </x:c>
       <x:c r="H14" s="28" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="I14" s="28" t="str"/>
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I14" s="28"/>
       <x:c r="J14" s="28" t="str">
-        <x:v>WBS 7.8</x:v>
+        <x:v>WBS 7.8 is integrated. Audit Record tests are ready for execution.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -7753,9 +7932,1289 @@
       <x:c r="H16" s="28" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="I16" s="28" t="str"/>
+      <x:c r="I16" s="28"/>
       <x:c r="J16" s="28" t="str">
-        <x:v>Final integration gate</x:v>
+        <x:v>Final integrated regression remains gated by unfinished WBS 7.7.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>S4-EV-AUTH-001</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="str">
+        <x:v>S4-AUTH-04; S4-AUTH-05</x:v>
+      </x:c>
+      <x:c r="C17" s="28" t="str">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="D17" s="28" t="str">
+        <x:v>Postman screenshots</x:v>
+      </x:c>
+      <x:c r="E17" s="28" t="str">
+        <x:v>Authentication rejection and authenticated current-user retrieval evidence</x:v>
+      </x:c>
+      <x:c r="F17" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AUTH-04_JWT_Protected_API_Without_Token_PASS.png; docs/testing/evidence/sprint-4/S4-AUTH-05_Current_User_Retrieval_After_Login_PASS.png</x:v>
+      </x:c>
+      <x:c r="G17" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I17" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J17" s="28" t="str">
+        <x:v>Both executed tests passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>S4-EV-PROFILE-001</x:v>
+      </x:c>
+      <x:c r="B18" s="28" t="str">
+        <x:v>S4-PROFILE-04</x:v>
+      </x:c>
+      <x:c r="C18" s="28" t="str">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="D18" s="28" t="str">
+        <x:v>Frontend screenshots</x:v>
+      </x:c>
+      <x:c r="E18" s="28" t="str">
+        <x:v>Profile change propagates to downstream Job Matching and baseline is restored</x:v>
+      </x:c>
+      <x:c r="F18" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-PROFILE-04_Profile_Baseline_Before_Skill_Change.png; docs/testing/evidence/sprint-4/S4-PROFILE-04_Job_Matching_Baseline_React_In_Profile.png; docs/testing/evidence/sprint-4/S4-PROFILE-04_Job_Matching_After_React_Removal_PASS.png; docs/testing/evidence/sprint-4/S4-PROFILE-04_Profile_Restored_React_Proficient_Verified.png</x:v>
+      </x:c>
+      <x:c r="G18" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H18" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I18" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J18" s="28" t="str">
+        <x:v>Executed test passed and React was restored at Proficient.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>S4-EV-REC-001</x:v>
+      </x:c>
+      <x:c r="B19" s="28" t="str">
+        <x:v>S4-REC-01</x:v>
+      </x:c>
+      <x:c r="C19" s="28" t="str">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="D19" s="28" t="str">
+        <x:v>Frontend screenshot</x:v>
+      </x:c>
+      <x:c r="E19" s="28" t="str">
+        <x:v>Ranked Career Recommendations result</x:v>
+      </x:c>
+      <x:c r="F19" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-REC-01_Ranked_Career_Recommendations_PASS.png</x:v>
+      </x:c>
+      <x:c r="G19" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H19" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I19" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J19" s="28" t="str">
+        <x:v>Executed test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>S4-EV-REC-003</x:v>
+      </x:c>
+      <x:c r="B20" s="28" t="str">
+        <x:v>S4-REC-03</x:v>
+      </x:c>
+      <x:c r="C20" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D20" s="28" t="str">
+        <x:v>Postman + frontend screenshots</x:v>
+      </x:c>
+      <x:c r="E20" s="28" t="str">
+        <x:v>AI recommendation explanation plus unchanged deterministic rank and score</x:v>
+      </x:c>
+      <x:c r="F20" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-REC-03_AI_Recommendation_Explanation_200_OK.png; docs/testing/evidence/sprint-4/S4-REC-03_Recommendation_Rank_and_Score_Unchanged_PASS.png</x:v>
+      </x:c>
+      <x:c r="G20" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H20" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I20" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J20" s="28" t="str">
+        <x:v>Executed test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>S4-EV-REC-004</x:v>
+      </x:c>
+      <x:c r="B21" s="28" t="str">
+        <x:v>S4-REC-04</x:v>
+      </x:c>
+      <x:c r="C21" s="28" t="str">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="D21" s="28" t="str">
+        <x:v>Postman assertions</x:v>
+      </x:c>
+      <x:c r="E21" s="28" t="str">
+        <x:v>Recommendation repeatability under unchanged Student Profile</x:v>
+      </x:c>
+      <x:c r="F21" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-REC-04_Recommendation_Repeatability_PASS.png</x:v>
+      </x:c>
+      <x:c r="G21" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H21" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I21" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J21" s="28" t="str">
+        <x:v>Postman full-array comparison passed 3/3.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>S4-EV-REC-006</x:v>
+      </x:c>
+      <x:c r="B22" s="28" t="str">
+        <x:v>S4-REC-06</x:v>
+      </x:c>
+      <x:c r="C22" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D22" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E22" s="28" t="str">
+        <x:v>AI explanation failure preserves deterministic recommendation payload</x:v>
+      </x:c>
+      <x:c r="F22" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-REC-06_AI_Explanation_Failure_Preserves_Recommendation_PASS.png</x:v>
+      </x:c>
+      <x:c r="G22" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H22" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I22" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J22" s="28" t="str">
+        <x:v>Existing backend regression test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>S4-EV-GAP-003</x:v>
+      </x:c>
+      <x:c r="B23" s="28" t="str">
+        <x:v>S4-GAP-03</x:v>
+      </x:c>
+      <x:c r="C23" s="28" t="str">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="D23" s="28" t="str">
+        <x:v>Postman assertions</x:v>
+      </x:c>
+      <x:c r="E23" s="28" t="str">
+        <x:v>Skill Gap and Career Readiness repeatability</x:v>
+      </x:c>
+      <x:c r="F23" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-GAP-03_Skill_Gap_Readiness_Repeatability_PASS.png</x:v>
+      </x:c>
+      <x:c r="G23" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H23" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I23" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J23" s="28" t="str">
+        <x:v>Postman deterministic comparison passed 4/4.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>S4-EV-GAP-004</x:v>
+      </x:c>
+      <x:c r="B24" s="28" t="str">
+        <x:v>S4-GAP-04</x:v>
+      </x:c>
+      <x:c r="C24" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D24" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E24" s="28" t="str">
+        <x:v>AI summary failure preserves deterministic Skill Gap and readiness</x:v>
+      </x:c>
+      <x:c r="F24" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-GAP-04_AI_Summary_Failure_Preserves_Skill_Gap_Readiness_PASS.png</x:v>
+      </x:c>
+      <x:c r="G24" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H24" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I24" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J24" s="28" t="str">
+        <x:v>Existing backend regression test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>S4-EV-GAP-005</x:v>
+      </x:c>
+      <x:c r="B25" s="28" t="str">
+        <x:v>S4-GAP-05</x:v>
+      </x:c>
+      <x:c r="C25" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D25" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E25" s="28" t="str">
+        <x:v>Readiness remains independent of text AI provider</x:v>
+      </x:c>
+      <x:c r="F25" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-GAP-05_Readiness_Independent_of_Text_AI_Provider_PASS.png</x:v>
+      </x:c>
+      <x:c r="G25" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H25" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I25" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J25" s="28" t="str">
+        <x:v>Existing backend regression test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>S4-EV-JOB-002</x:v>
+      </x:c>
+      <x:c r="B26" s="28" t="str">
+        <x:v>S4-JOB-02</x:v>
+      </x:c>
+      <x:c r="C26" s="28" t="str">
+        <x:v>7.2,7.5,7.9</x:v>
+      </x:c>
+      <x:c r="D26" s="28" t="str">
+        <x:v>Frontend screenshot</x:v>
+      </x:c>
+      <x:c r="E26" s="28" t="str">
+        <x:v>Valid job description returns matched and missing requirements</x:v>
+      </x:c>
+      <x:c r="F26" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-02_Valid_Job_Description_Matched_Missing_Requirements_PASS.png</x:v>
+      </x:c>
+      <x:c r="G26" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H26" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I26" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J26" s="28" t="str">
+        <x:v>Executed test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>S4-EV-JOB-003</x:v>
+      </x:c>
+      <x:c r="B27" s="28" t="str">
+        <x:v>S4-JOB-03</x:v>
+      </x:c>
+      <x:c r="C27" s="28" t="str">
+        <x:v>7.2,7.5,7.9</x:v>
+      </x:c>
+      <x:c r="D27" s="28" t="str">
+        <x:v>Frontend screenshot</x:v>
+      </x:c>
+      <x:c r="E27" s="28" t="str">
+        <x:v>Blank job-description validation</x:v>
+      </x:c>
+      <x:c r="F27" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-03_Blank_Job_Description_Validation_PASS.png</x:v>
+      </x:c>
+      <x:c r="G27" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H27" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I27" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J27" s="28" t="str">
+        <x:v>Executed test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>S4-EV-JOB-004</x:v>
+      </x:c>
+      <x:c r="B28" s="28" t="str">
+        <x:v>S4-JOB-04</x:v>
+      </x:c>
+      <x:c r="C28" s="28" t="str">
+        <x:v>7.2,7.5,7.9</x:v>
+      </x:c>
+      <x:c r="D28" s="28" t="str">
+        <x:v>Frontend screenshot</x:v>
+      </x:c>
+      <x:c r="E28" s="28" t="str">
+        <x:v>Oversized job-description validation</x:v>
+      </x:c>
+      <x:c r="F28" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-04_Oversized_Job_Description_Validation_PASS.png</x:v>
+      </x:c>
+      <x:c r="G28" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H28" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I28" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J28" s="28" t="str">
+        <x:v>Executed test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>S4-EV-JOB-007</x:v>
+      </x:c>
+      <x:c r="B29" s="28" t="str">
+        <x:v>S4-JOB-07</x:v>
+      </x:c>
+      <x:c r="C29" s="28" t="str">
+        <x:v>7.2,7.9</x:v>
+      </x:c>
+      <x:c r="D29" s="28" t="str">
+        <x:v>Frontend screenshot</x:v>
+      </x:c>
+      <x:c r="E29" s="28" t="str">
+        <x:v>Canonical Skill matching for React</x:v>
+      </x:c>
+      <x:c r="F29" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-07_Canonical_Skill_Matching_React_PASS.png</x:v>
+      </x:c>
+      <x:c r="G29" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H29" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I29" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J29" s="28" t="str">
+        <x:v>Executed test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>S4-EV-JOB-008</x:v>
+      </x:c>
+      <x:c r="B30" s="28" t="str">
+        <x:v>S4-JOB-08</x:v>
+      </x:c>
+      <x:c r="C30" s="28" t="str">
+        <x:v>7.2,7.9</x:v>
+      </x:c>
+      <x:c r="D30" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E30" s="28" t="str">
+        <x:v>SkillAlias Py resolves to canonical Python Skill</x:v>
+      </x:c>
+      <x:c r="F30" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-08_Skill_Alias_Matching_Py_to_Python_PASS.png</x:v>
+      </x:c>
+      <x:c r="G30" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H30" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I30" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J30" s="28" t="str">
+        <x:v>Existing backend test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>S4-EV-JOB-009</x:v>
+      </x:c>
+      <x:c r="B31" s="28" t="str">
+        <x:v>S4-JOB-09</x:v>
+      </x:c>
+      <x:c r="C31" s="28" t="str">
+        <x:v>7.2,7.9</x:v>
+      </x:c>
+      <x:c r="D31" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E31" s="28" t="str">
+        <x:v>Unsupported related wording is not guessed</x:v>
+      </x:c>
+      <x:c r="F31" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-09_Unsupported_Synonym_Guessing_Not_Guessed_PASS.png</x:v>
+      </x:c>
+      <x:c r="G31" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H31" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I31" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J31" s="28" t="str">
+        <x:v>Existing backend test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>S4-EV-JOB-010</x:v>
+      </x:c>
+      <x:c r="B32" s="28" t="str">
+        <x:v>S4-JOB-10</x:v>
+      </x:c>
+      <x:c r="C32" s="28" t="str">
+        <x:v>7.2,7.9</x:v>
+      </x:c>
+      <x:c r="D32" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E32" s="28" t="str">
+        <x:v>Generic Design false positive is avoided</x:v>
+      </x:c>
+      <x:c r="F32" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-10_Generic_Design_False_Positive_Avoided_PASS.png</x:v>
+      </x:c>
+      <x:c r="G32" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H32" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I32" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J32" s="28" t="str">
+        <x:v>Existing backend test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>S4-EV-JOB-011</x:v>
+      </x:c>
+      <x:c r="B33" s="28" t="str">
+        <x:v>S4-JOB-11</x:v>
+      </x:c>
+      <x:c r="C33" s="28" t="str">
+        <x:v>7.2,7.9</x:v>
+      </x:c>
+      <x:c r="D33" s="28" t="str">
+        <x:v>API contract + UI evidence</x:v>
+      </x:c>
+      <x:c r="E33" s="28" t="str">
+        <x:v>Job Matching does not expose hiring probability or suitability score</x:v>
+      </x:c>
+      <x:c r="F33" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-11_No_Suitability_Score_API_Contract_PASS.png; docs/testing/evidence/sprint-4/S4-JOB-02_Valid_Job_Description_Matched_Missing_Requirements_PASS.png</x:v>
+      </x:c>
+      <x:c r="G33" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H33" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I33" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J33" s="28" t="str">
+        <x:v>API contract passed and UI states result is not an employment suitability score.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>S4-EV-JOB-012</x:v>
+      </x:c>
+      <x:c r="B34" s="28" t="str">
+        <x:v>S4-JOB-12</x:v>
+      </x:c>
+      <x:c r="C34" s="28" t="str">
+        <x:v>7.2,7.9</x:v>
+      </x:c>
+      <x:c r="D34" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E34" s="28" t="str">
+        <x:v>Unsupported client ownership override is rejected</x:v>
+      </x:c>
+      <x:c r="F34" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-12_Reject_Client_Ownership_Override_PASS.png</x:v>
+      </x:c>
+      <x:c r="G34" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H34" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I34" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J34" s="28" t="str">
+        <x:v>Existing backend ownership test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>S4-EV-JOB-013</x:v>
+      </x:c>
+      <x:c r="B35" s="28" t="str">
+        <x:v>S4-JOB-13</x:v>
+      </x:c>
+      <x:c r="C35" s="28" t="str">
+        <x:v>7.2,7.9</x:v>
+      </x:c>
+      <x:c r="D35" s="28" t="str">
+        <x:v>Frontend screenshot</x:v>
+      </x:c>
+      <x:c r="E35" s="28" t="str">
+        <x:v>Job Matching does not mutate Student Profile</x:v>
+      </x:c>
+      <x:c r="F35" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-JOB-13_Job_Matching_Does_Not_Mutate_Profile_PASS.png</x:v>
+      </x:c>
+      <x:c r="G35" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H35" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I35" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J35" s="28" t="str">
+        <x:v>Profile baseline remained unchanged after Job Matching operations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>S4-EV-RESUME-005</x:v>
+      </x:c>
+      <x:c r="B36" s="28" t="str">
+        <x:v>S4-RESUME-05</x:v>
+      </x:c>
+      <x:c r="C36" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D36" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E36" s="28" t="str">
+        <x:v>Resume provider failure is controlled</x:v>
+      </x:c>
+      <x:c r="F36" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-RESUME-05_Resume_Provider_Failure_Controlled_PASS.png</x:v>
+      </x:c>
+      <x:c r="G36" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H36" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I36" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J36" s="28" t="str">
+        <x:v>Provider unavailable path returned controlled 503.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>S4-EV-RESUME-006</x:v>
+      </x:c>
+      <x:c r="B37" s="28" t="str">
+        <x:v>S4-RESUME-06</x:v>
+      </x:c>
+      <x:c r="C37" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D37" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E37" s="28" t="str">
+        <x:v>Resume invalid AI response is rejected and sanitized</x:v>
+      </x:c>
+      <x:c r="F37" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-RESUME-06_Invalid_AI_Response_Rejected_PASS.png</x:v>
+      </x:c>
+      <x:c r="G37" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H37" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I37" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J37" s="28" t="str">
+        <x:v>Response-validation failure returned sanitized 503.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>S4-EV-COVER-006</x:v>
+      </x:c>
+      <x:c r="B38" s="28" t="str">
+        <x:v>S4-COVER-06</x:v>
+      </x:c>
+      <x:c r="C38" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D38" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E38" s="28" t="str">
+        <x:v>Cover Letter provider failure is controlled</x:v>
+      </x:c>
+      <x:c r="F38" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-COVER-06_Cover_Letter_Provider_Failure_Controlled_PASS.png</x:v>
+      </x:c>
+      <x:c r="G38" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H38" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I38" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J38" s="28" t="str">
+        <x:v>Provider unavailable path returned controlled 503.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>S4-EV-INT-002</x:v>
+      </x:c>
+      <x:c r="B39" s="28" t="str">
+        <x:v>S4-INT-02</x:v>
+      </x:c>
+      <x:c r="C39" s="28" t="str">
+        <x:v>7.3,7.9</x:v>
+      </x:c>
+      <x:c r="D39" s="28" t="str">
+        <x:v>Postman screenshot</x:v>
+      </x:c>
+      <x:c r="E39" s="28" t="str">
+        <x:v>Valid Interview Questions request returns structured questions</x:v>
+      </x:c>
+      <x:c r="F39" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-INT-02_Generate_Valid_Interview_Questions_PASS.png</x:v>
+      </x:c>
+      <x:c r="G39" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H39" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I39" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J39" s="28" t="str">
+        <x:v>Five role-relevant questions returned with HTTP 200.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>S4-EV-INT-003</x:v>
+      </x:c>
+      <x:c r="B40" s="28" t="str">
+        <x:v>S4-INT-03</x:v>
+      </x:c>
+      <x:c r="C40" s="28" t="str">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="D40" s="28" t="str">
+        <x:v>Postman screenshot</x:v>
+      </x:c>
+      <x:c r="E40" s="28" t="str">
+        <x:v>Question count below minimum is rejected</x:v>
+      </x:c>
+      <x:c r="F40" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-INT-03_Reject_Question_Count_Below_Range_PASS.png</x:v>
+      </x:c>
+      <x:c r="G40" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H40" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I40" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J40" s="28" t="str">
+        <x:v>question_count=0 returned controlled validation error.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>S4-EV-INT-004</x:v>
+      </x:c>
+      <x:c r="B41" s="28" t="str">
+        <x:v>S4-INT-04</x:v>
+      </x:c>
+      <x:c r="C41" s="28" t="str">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="D41" s="28" t="str">
+        <x:v>Postman screenshot</x:v>
+      </x:c>
+      <x:c r="E41" s="28" t="str">
+        <x:v>Question count above maximum is rejected</x:v>
+      </x:c>
+      <x:c r="F41" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-INT-04_Reject_Question_Count_Above_Range_PASS.png</x:v>
+      </x:c>
+      <x:c r="G41" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H41" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I41" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J41" s="28" t="str">
+        <x:v>question_count=11 returned controlled validation error.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>S4-EV-INT-007</x:v>
+      </x:c>
+      <x:c r="B42" s="28" t="str">
+        <x:v>S4-INT-07</x:v>
+      </x:c>
+      <x:c r="C42" s="28" t="str">
+        <x:v>7.3,7.9</x:v>
+      </x:c>
+      <x:c r="D42" s="28" t="str">
+        <x:v>Postman screenshot</x:v>
+      </x:c>
+      <x:c r="E42" s="28" t="str">
+        <x:v>Structured Interview Feedback is generated</x:v>
+      </x:c>
+      <x:c r="F42" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-INT-07_Generate_Structured_Interview_Feedback_PASS.png</x:v>
+      </x:c>
+      <x:c r="G42" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H42" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I42" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J42" s="28" t="str">
+        <x:v>Structured strengths, improvements and suggested response returned.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>S4-EV-INT-008</x:v>
+      </x:c>
+      <x:c r="B43" s="28" t="str">
+        <x:v>S4-INT-08</x:v>
+      </x:c>
+      <x:c r="C43" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D43" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E43" s="28" t="str">
+        <x:v>Semantically invalid focus areas are rejected</x:v>
+      </x:c>
+      <x:c r="F43" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-INT-08_Reject_Semantically_Invalid_Focus_Areas_PASS.png</x:v>
+      </x:c>
+      <x:c r="G43" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H43" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I43" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J43" s="28" t="str">
+        <x:v>Controlled 502 semantic validation path passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>S4-EV-INT-009</x:v>
+      </x:c>
+      <x:c r="B44" s="28" t="str">
+        <x:v>S4-INT-09</x:v>
+      </x:c>
+      <x:c r="C44" s="28" t="str">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="D44" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E44" s="28" t="str">
+        <x:v>Interview outputs exclude hiring probability and pass-fail classification</x:v>
+      </x:c>
+      <x:c r="F44" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-INT-09_Exclude_Hiring_Probability_Pass_Fail_PASS.png</x:v>
+      </x:c>
+      <x:c r="G44" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H44" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I44" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J44" s="28" t="str">
+        <x:v>Question and feedback response-contract tests both passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>S4-EV-AI-CASE-001</x:v>
+      </x:c>
+      <x:c r="B45" s="28" t="str">
+        <x:v>S4-AI-01</x:v>
+      </x:c>
+      <x:c r="C45" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D45" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E45" s="28" t="str">
+        <x:v>Completed valid AI response is accepted</x:v>
+      </x:c>
+      <x:c r="F45" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-01_Accept_Completed_AI_Response_PASS.png</x:v>
+      </x:c>
+      <x:c r="G45" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H45" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I45" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J45" s="28" t="str">
+        <x:v>Provider validation test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>S4-EV-AI-CASE-002</x:v>
+      </x:c>
+      <x:c r="B46" s="28" t="str">
+        <x:v>S4-AI-02</x:v>
+      </x:c>
+      <x:c r="C46" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D46" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E46" s="28" t="str">
+        <x:v>Incomplete AI response is rejected</x:v>
+      </x:c>
+      <x:c r="F46" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-02_Reject_Incomplete_AI_Response_PASS.png</x:v>
+      </x:c>
+      <x:c r="G46" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H46" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I46" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J46" s="28" t="str">
+        <x:v>Provider validation test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>S4-EV-AI-CASE-003</x:v>
+      </x:c>
+      <x:c r="B47" s="28" t="str">
+        <x:v>S4-AI-03</x:v>
+      </x:c>
+      <x:c r="C47" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D47" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E47" s="28" t="str">
+        <x:v>Failed AI response state is rejected</x:v>
+      </x:c>
+      <x:c r="F47" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-03-05_Reject_Non_Completed_AI_Response_States_PASS.png</x:v>
+      </x:c>
+      <x:c r="G47" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H47" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I47" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J47" s="28" t="str">
+        <x:v>Shared non-completed-state test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>S4-EV-AI-CASE-004</x:v>
+      </x:c>
+      <x:c r="B48" s="28" t="str">
+        <x:v>S4-AI-04</x:v>
+      </x:c>
+      <x:c r="C48" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D48" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E48" s="28" t="str">
+        <x:v>Cancelled AI response state is rejected</x:v>
+      </x:c>
+      <x:c r="F48" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-03-05_Reject_Non_Completed_AI_Response_States_PASS.png</x:v>
+      </x:c>
+      <x:c r="G48" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H48" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I48" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J48" s="28" t="str">
+        <x:v>Shared non-completed-state test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>S4-EV-AI-CASE-005</x:v>
+      </x:c>
+      <x:c r="B49" s="28" t="str">
+        <x:v>S4-AI-05</x:v>
+      </x:c>
+      <x:c r="C49" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D49" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E49" s="28" t="str">
+        <x:v>Queued and in-progress AI response states are rejected</x:v>
+      </x:c>
+      <x:c r="F49" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-03-05_Reject_Non_Completed_AI_Response_States_PASS.png</x:v>
+      </x:c>
+      <x:c r="G49" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H49" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I49" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J49" s="28" t="str">
+        <x:v>Shared non-completed-state test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>S4-EV-AI-CASE-006</x:v>
+      </x:c>
+      <x:c r="B50" s="28" t="str">
+        <x:v>S4-AI-06</x:v>
+      </x:c>
+      <x:c r="C50" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D50" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E50" s="28" t="str">
+        <x:v>Missing AI response status is rejected</x:v>
+      </x:c>
+      <x:c r="F50" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-06_Reject_Missing_AI_Response_Status_PASS.png</x:v>
+      </x:c>
+      <x:c r="G50" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H50" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I50" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J50" s="28" t="str">
+        <x:v>Provider validation test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>S4-EV-AI-CASE-007</x:v>
+      </x:c>
+      <x:c r="B51" s="28" t="str">
+        <x:v>S4-AI-07</x:v>
+      </x:c>
+      <x:c r="C51" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D51" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E51" s="28" t="str">
+        <x:v>Completed AI response with empty output is rejected</x:v>
+      </x:c>
+      <x:c r="F51" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-07_Reject_Empty_AI_Output_PASS.png</x:v>
+      </x:c>
+      <x:c r="G51" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H51" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I51" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J51" s="28" t="str">
+        <x:v>Structured-output validation test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>S4-EV-AI-CASE-008</x:v>
+      </x:c>
+      <x:c r="B52" s="28" t="str">
+        <x:v>S4-AI-08</x:v>
+      </x:c>
+      <x:c r="C52" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D52" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E52" s="28" t="str">
+        <x:v>Malformed AI JSON is rejected</x:v>
+      </x:c>
+      <x:c r="F52" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-08_Reject_Malformed_AI_JSON_PASS.png</x:v>
+      </x:c>
+      <x:c r="G52" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H52" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I52" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J52" s="28" t="str">
+        <x:v>Structured-output validation test passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>S4-EV-AI-CASE-009</x:v>
+      </x:c>
+      <x:c r="B53" s="28" t="str">
+        <x:v>S4-AI-09</x:v>
+      </x:c>
+      <x:c r="C53" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D53" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E53" s="28" t="str">
+        <x:v>Provider timeout is translated safely</x:v>
+      </x:c>
+      <x:c r="F53" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-09_Translate_Provider_Timeout_Safely_PASS.png</x:v>
+      </x:c>
+      <x:c r="G53" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H53" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I53" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J53" s="28" t="str">
+        <x:v>Provider timeout details were not exposed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>S4-EV-AI-CASE-010</x:v>
+      </x:c>
+      <x:c r="B54" s="28" t="str">
+        <x:v>S4-AI-10</x:v>
+      </x:c>
+      <x:c r="C54" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D54" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E54" s="28" t="str">
+        <x:v>Provider connection failure is translated safely</x:v>
+      </x:c>
+      <x:c r="F54" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-10_Translate_Connection_Failure_Safely_PASS.png</x:v>
+      </x:c>
+      <x:c r="G54" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H54" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I54" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J54" s="28" t="str">
+        <x:v>Connection failure details were sanitized.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>S4-EV-AI-CASE-011</x:v>
+      </x:c>
+      <x:c r="B55" s="28" t="str">
+        <x:v>S4-AI-11</x:v>
+      </x:c>
+      <x:c r="C55" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D55" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E55" s="28" t="str">
+        <x:v>Rate-limit and HTTP provider failures are translated safely</x:v>
+      </x:c>
+      <x:c r="F55" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-11_Translate_Rate_Limit_HTTP_Failure_Safely_PASS.png</x:v>
+      </x:c>
+      <x:c r="G55" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H55" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I55" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J55" s="28" t="str">
+        <x:v>Rate-limit and HTTP status failure tests passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>S4-EV-AI-CASE-012</x:v>
+      </x:c>
+      <x:c r="B56" s="28" t="str">
+        <x:v>S4-AI-12</x:v>
+      </x:c>
+      <x:c r="C56" s="28" t="str">
+        <x:v>7.4,7.9</x:v>
+      </x:c>
+      <x:c r="D56" s="28" t="str">
+        <x:v>Automated terminal output</x:v>
+      </x:c>
+      <x:c r="E56" s="28" t="str">
+        <x:v>Deterministic results remain protected during AI failure</x:v>
+      </x:c>
+      <x:c r="F56" s="28" t="str">
+        <x:v>docs/testing/evidence/sprint-4/S4-AI-12_Protect_Deterministic_Results_During_AI_Failure_PASS.png</x:v>
+      </x:c>
+      <x:c r="G56" s="28" t="str">
+        <x:v>Jerald</x:v>
+      </x:c>
+      <x:c r="H56" s="28" t="str">
+        <x:v>Captured</x:v>
+      </x:c>
+      <x:c r="I56" s="28" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="J56" s="28" t="str">
+        <x:v>Recommendation, Skill Gap, Readiness and Job Matching protection tests passed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7770,7 +9229,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b8b3ea5bf074d0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b60b38862b84acb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>